<commit_message>
feat: agregar fotos 44 y 45 - Donita Juan Camilo y Alejandra
Donita Juan Camilo (BJK95I): 24 meses, tarifa 420.000/mes MENSUAL, 4 pagos
Alejandra (OKS30I): 21 meses / 84 cuotas, 13 pagos semanales abr-jul 2026
Ambos clientes anadidos a cobro_index.html y Excel regenerado

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/control_motos_tio.xlsx
+++ b/control_motos_tio.xlsx
@@ -565,7 +565,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F22"/>
+  <dimension ref="A1:F28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -1196,6 +1196,174 @@
         <v>84</v>
       </c>
     </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Ana Milena Juan Davit</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Bajaj UPY 65H</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>UPY65H</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="n">
+        <v>46045</v>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Foto 40 | 25 pagos registrados | cuotas pendientes a confirmar</t>
+        </is>
+      </c>
+      <c r="F23" t="n">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Sr Luis</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Bajaj UYZ 32H</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>UYZ32H</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="n">
+        <v>46027</v>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Foto 41 | 14 pagos registrados | nota: calibrar moto</t>
+        </is>
+      </c>
+      <c r="F24" t="n">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Manuel Alga</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Bajaj UYZ 39H</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>UYZ39H</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="n">
+        <v>46065</v>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Foto 42 | 18 meses | 72 cuotas | 18 pagos registrados</t>
+        </is>
+      </c>
+      <c r="F25" t="n">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Jorge Estrada</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Bajaj BJH 66I</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>BJH66I</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="n">
+        <v>46069</v>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Foto 43 | 64 cuotas | 18 meses | 16 pagos | GAP en mayo-2026 sin registro</t>
+        </is>
+      </c>
+      <c r="F26" t="n">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Donita Juan Camilo</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Bajaj BJK 95I</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>BJK95I</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="n">
+        <v>46086</v>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Foto 44 | 24 meses | 24 cuotas MENSUALES | tarifa 420.000/mes | total 10.080.000</t>
+        </is>
+      </c>
+      <c r="F27" t="n">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Alejandra</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Bajaj OKS 30I</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>OKS30I</t>
+        </is>
+      </c>
+      <c r="D28" s="2" t="n">
+        <v>46123</v>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Foto 45 | 21 meses | 84 cuotas | 13 pagos registrados</t>
+        </is>
+      </c>
+      <c r="F28" t="n">
+        <v>84</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1207,7 +1375,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P998"/>
+  <dimension ref="A1:P1088"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -32177,6 +32345,2796 @@
         <v>240000</v>
       </c>
       <c r="J998" t="inlineStr">
+        <is>
+          <t>efectivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="999">
+      <c r="A999" s="3" t="n">
+        <v>46045</v>
+      </c>
+      <c r="B999" t="inlineStr">
+        <is>
+          <t>Ana Milena Juan Davit</t>
+        </is>
+      </c>
+      <c r="C999" t="inlineStr">
+        <is>
+          <t>Bajaj UPY 65H</t>
+        </is>
+      </c>
+      <c r="D999" t="inlineStr">
+        <is>
+          <t>UPY65H</t>
+        </is>
+      </c>
+      <c r="H999" t="n">
+        <v>240000</v>
+      </c>
+      <c r="I999" t="n">
+        <v>240000</v>
+      </c>
+      <c r="J999" t="inlineStr">
+        <is>
+          <t>efectivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="1000">
+      <c r="A1000" s="3" t="n">
+        <v>46054</v>
+      </c>
+      <c r="B1000" t="inlineStr">
+        <is>
+          <t>Ana Milena Juan Davit</t>
+        </is>
+      </c>
+      <c r="C1000" t="inlineStr">
+        <is>
+          <t>Bajaj UPY 65H</t>
+        </is>
+      </c>
+      <c r="D1000" t="inlineStr">
+        <is>
+          <t>UPY65H</t>
+        </is>
+      </c>
+      <c r="H1000" t="n">
+        <v>240000</v>
+      </c>
+      <c r="I1000" t="n">
+        <v>240000</v>
+      </c>
+      <c r="J1000" t="inlineStr">
+        <is>
+          <t>efectivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="1001">
+      <c r="A1001" s="3" t="n">
+        <v>46064</v>
+      </c>
+      <c r="B1001" t="inlineStr">
+        <is>
+          <t>Ana Milena Juan Davit</t>
+        </is>
+      </c>
+      <c r="C1001" t="inlineStr">
+        <is>
+          <t>Bajaj UPY 65H</t>
+        </is>
+      </c>
+      <c r="D1001" t="inlineStr">
+        <is>
+          <t>UPY65H</t>
+        </is>
+      </c>
+      <c r="H1001" t="n">
+        <v>240000</v>
+      </c>
+      <c r="I1001" t="n">
+        <v>240000</v>
+      </c>
+      <c r="J1001" t="inlineStr">
+        <is>
+          <t>efectivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="1002">
+      <c r="A1002" s="3" t="n">
+        <v>46071</v>
+      </c>
+      <c r="B1002" t="inlineStr">
+        <is>
+          <t>Ana Milena Juan Davit</t>
+        </is>
+      </c>
+      <c r="C1002" t="inlineStr">
+        <is>
+          <t>Bajaj UPY 65H</t>
+        </is>
+      </c>
+      <c r="D1002" t="inlineStr">
+        <is>
+          <t>UPY65H</t>
+        </is>
+      </c>
+      <c r="H1002" t="n">
+        <v>240000</v>
+      </c>
+      <c r="I1002" t="n">
+        <v>240000</v>
+      </c>
+      <c r="J1002" t="inlineStr">
+        <is>
+          <t>efectivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="1003">
+      <c r="A1003" s="3" t="n">
+        <v>46079</v>
+      </c>
+      <c r="B1003" t="inlineStr">
+        <is>
+          <t>Ana Milena Juan Davit</t>
+        </is>
+      </c>
+      <c r="C1003" t="inlineStr">
+        <is>
+          <t>Bajaj UPY 65H</t>
+        </is>
+      </c>
+      <c r="D1003" t="inlineStr">
+        <is>
+          <t>UPY65H</t>
+        </is>
+      </c>
+      <c r="H1003" t="n">
+        <v>240000</v>
+      </c>
+      <c r="I1003" t="n">
+        <v>240000</v>
+      </c>
+      <c r="J1003" t="inlineStr">
+        <is>
+          <t>efectivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="1004">
+      <c r="A1004" s="3" t="n">
+        <v>46086</v>
+      </c>
+      <c r="B1004" t="inlineStr">
+        <is>
+          <t>Ana Milena Juan Davit</t>
+        </is>
+      </c>
+      <c r="C1004" t="inlineStr">
+        <is>
+          <t>Bajaj UPY 65H</t>
+        </is>
+      </c>
+      <c r="D1004" t="inlineStr">
+        <is>
+          <t>UPY65H</t>
+        </is>
+      </c>
+      <c r="H1004" t="n">
+        <v>240000</v>
+      </c>
+      <c r="I1004" t="n">
+        <v>240000</v>
+      </c>
+      <c r="J1004" t="inlineStr">
+        <is>
+          <t>efectivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="1005">
+      <c r="A1005" s="3" t="n">
+        <v>46093</v>
+      </c>
+      <c r="B1005" t="inlineStr">
+        <is>
+          <t>Ana Milena Juan Davit</t>
+        </is>
+      </c>
+      <c r="C1005" t="inlineStr">
+        <is>
+          <t>Bajaj UPY 65H</t>
+        </is>
+      </c>
+      <c r="D1005" t="inlineStr">
+        <is>
+          <t>UPY65H</t>
+        </is>
+      </c>
+      <c r="H1005" t="n">
+        <v>240000</v>
+      </c>
+      <c r="I1005" t="n">
+        <v>240000</v>
+      </c>
+      <c r="J1005" t="inlineStr">
+        <is>
+          <t>efectivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="1006">
+      <c r="A1006" s="3" t="n">
+        <v>46100</v>
+      </c>
+      <c r="B1006" t="inlineStr">
+        <is>
+          <t>Ana Milena Juan Davit</t>
+        </is>
+      </c>
+      <c r="C1006" t="inlineStr">
+        <is>
+          <t>Bajaj UPY 65H</t>
+        </is>
+      </c>
+      <c r="D1006" t="inlineStr">
+        <is>
+          <t>UPY65H</t>
+        </is>
+      </c>
+      <c r="H1006" t="n">
+        <v>240000</v>
+      </c>
+      <c r="I1006" t="n">
+        <v>240000</v>
+      </c>
+      <c r="J1006" t="inlineStr">
+        <is>
+          <t>efectivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="1007">
+      <c r="A1007" s="3" t="n">
+        <v>46107</v>
+      </c>
+      <c r="B1007" t="inlineStr">
+        <is>
+          <t>Ana Milena Juan Davit</t>
+        </is>
+      </c>
+      <c r="C1007" t="inlineStr">
+        <is>
+          <t>Bajaj UPY 65H</t>
+        </is>
+      </c>
+      <c r="D1007" t="inlineStr">
+        <is>
+          <t>UPY65H</t>
+        </is>
+      </c>
+      <c r="H1007" t="n">
+        <v>240000</v>
+      </c>
+      <c r="I1007" t="n">
+        <v>240000</v>
+      </c>
+      <c r="J1007" t="inlineStr">
+        <is>
+          <t>efectivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="1008">
+      <c r="A1008" s="3" t="n">
+        <v>46114</v>
+      </c>
+      <c r="B1008" t="inlineStr">
+        <is>
+          <t>Ana Milena Juan Davit</t>
+        </is>
+      </c>
+      <c r="C1008" t="inlineStr">
+        <is>
+          <t>Bajaj UPY 65H</t>
+        </is>
+      </c>
+      <c r="D1008" t="inlineStr">
+        <is>
+          <t>UPY65H</t>
+        </is>
+      </c>
+      <c r="H1008" t="n">
+        <v>240000</v>
+      </c>
+      <c r="I1008" t="n">
+        <v>240000</v>
+      </c>
+      <c r="J1008" t="inlineStr">
+        <is>
+          <t>efectivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="1009">
+      <c r="A1009" s="3" t="n">
+        <v>46121</v>
+      </c>
+      <c r="B1009" t="inlineStr">
+        <is>
+          <t>Ana Milena Juan Davit</t>
+        </is>
+      </c>
+      <c r="C1009" t="inlineStr">
+        <is>
+          <t>Bajaj UPY 65H</t>
+        </is>
+      </c>
+      <c r="D1009" t="inlineStr">
+        <is>
+          <t>UPY65H</t>
+        </is>
+      </c>
+      <c r="H1009" t="n">
+        <v>240000</v>
+      </c>
+      <c r="I1009" t="n">
+        <v>240000</v>
+      </c>
+      <c r="J1009" t="inlineStr">
+        <is>
+          <t>efectivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="1010">
+      <c r="A1010" s="3" t="n">
+        <v>46128</v>
+      </c>
+      <c r="B1010" t="inlineStr">
+        <is>
+          <t>Ana Milena Juan Davit</t>
+        </is>
+      </c>
+      <c r="C1010" t="inlineStr">
+        <is>
+          <t>Bajaj UPY 65H</t>
+        </is>
+      </c>
+      <c r="D1010" t="inlineStr">
+        <is>
+          <t>UPY65H</t>
+        </is>
+      </c>
+      <c r="H1010" t="n">
+        <v>240000</v>
+      </c>
+      <c r="I1010" t="n">
+        <v>240000</v>
+      </c>
+      <c r="J1010" t="inlineStr">
+        <is>
+          <t>efectivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="1011">
+      <c r="A1011" s="3" t="n">
+        <v>46135</v>
+      </c>
+      <c r="B1011" t="inlineStr">
+        <is>
+          <t>Ana Milena Juan Davit</t>
+        </is>
+      </c>
+      <c r="C1011" t="inlineStr">
+        <is>
+          <t>Bajaj UPY 65H</t>
+        </is>
+      </c>
+      <c r="D1011" t="inlineStr">
+        <is>
+          <t>UPY65H</t>
+        </is>
+      </c>
+      <c r="H1011" t="n">
+        <v>240000</v>
+      </c>
+      <c r="I1011" t="n">
+        <v>240000</v>
+      </c>
+      <c r="J1011" t="inlineStr">
+        <is>
+          <t>efectivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="1012">
+      <c r="A1012" s="3" t="n">
+        <v>46142</v>
+      </c>
+      <c r="B1012" t="inlineStr">
+        <is>
+          <t>Ana Milena Juan Davit</t>
+        </is>
+      </c>
+      <c r="C1012" t="inlineStr">
+        <is>
+          <t>Bajaj UPY 65H</t>
+        </is>
+      </c>
+      <c r="D1012" t="inlineStr">
+        <is>
+          <t>UPY65H</t>
+        </is>
+      </c>
+      <c r="H1012" t="n">
+        <v>240000</v>
+      </c>
+      <c r="I1012" t="n">
+        <v>240000</v>
+      </c>
+      <c r="J1012" t="inlineStr">
+        <is>
+          <t>efectivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="1013">
+      <c r="A1013" s="3" t="n">
+        <v>46149</v>
+      </c>
+      <c r="B1013" t="inlineStr">
+        <is>
+          <t>Ana Milena Juan Davit</t>
+        </is>
+      </c>
+      <c r="C1013" t="inlineStr">
+        <is>
+          <t>Bajaj UPY 65H</t>
+        </is>
+      </c>
+      <c r="D1013" t="inlineStr">
+        <is>
+          <t>UPY65H</t>
+        </is>
+      </c>
+      <c r="H1013" t="n">
+        <v>240000</v>
+      </c>
+      <c r="I1013" t="n">
+        <v>240000</v>
+      </c>
+      <c r="J1013" t="inlineStr">
+        <is>
+          <t>efectivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="1014">
+      <c r="A1014" s="3" t="n">
+        <v>46156</v>
+      </c>
+      <c r="B1014" t="inlineStr">
+        <is>
+          <t>Ana Milena Juan Davit</t>
+        </is>
+      </c>
+      <c r="C1014" t="inlineStr">
+        <is>
+          <t>Bajaj UPY 65H</t>
+        </is>
+      </c>
+      <c r="D1014" t="inlineStr">
+        <is>
+          <t>UPY65H</t>
+        </is>
+      </c>
+      <c r="H1014" t="n">
+        <v>240000</v>
+      </c>
+      <c r="I1014" t="n">
+        <v>240000</v>
+      </c>
+      <c r="J1014" t="inlineStr">
+        <is>
+          <t>efectivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="1015">
+      <c r="A1015" s="3" t="n">
+        <v>46163</v>
+      </c>
+      <c r="B1015" t="inlineStr">
+        <is>
+          <t>Ana Milena Juan Davit</t>
+        </is>
+      </c>
+      <c r="C1015" t="inlineStr">
+        <is>
+          <t>Bajaj UPY 65H</t>
+        </is>
+      </c>
+      <c r="D1015" t="inlineStr">
+        <is>
+          <t>UPY65H</t>
+        </is>
+      </c>
+      <c r="H1015" t="n">
+        <v>240000</v>
+      </c>
+      <c r="I1015" t="n">
+        <v>240000</v>
+      </c>
+      <c r="J1015" t="inlineStr">
+        <is>
+          <t>efectivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="1016">
+      <c r="A1016" s="3" t="n">
+        <v>46170</v>
+      </c>
+      <c r="B1016" t="inlineStr">
+        <is>
+          <t>Ana Milena Juan Davit</t>
+        </is>
+      </c>
+      <c r="C1016" t="inlineStr">
+        <is>
+          <t>Bajaj UPY 65H</t>
+        </is>
+      </c>
+      <c r="D1016" t="inlineStr">
+        <is>
+          <t>UPY65H</t>
+        </is>
+      </c>
+      <c r="H1016" t="n">
+        <v>240000</v>
+      </c>
+      <c r="I1016" t="n">
+        <v>240000</v>
+      </c>
+      <c r="J1016" t="inlineStr">
+        <is>
+          <t>efectivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="1017">
+      <c r="A1017" s="3" t="n">
+        <v>46177</v>
+      </c>
+      <c r="B1017" t="inlineStr">
+        <is>
+          <t>Ana Milena Juan Davit</t>
+        </is>
+      </c>
+      <c r="C1017" t="inlineStr">
+        <is>
+          <t>Bajaj UPY 65H</t>
+        </is>
+      </c>
+      <c r="D1017" t="inlineStr">
+        <is>
+          <t>UPY65H</t>
+        </is>
+      </c>
+      <c r="H1017" t="n">
+        <v>240000</v>
+      </c>
+      <c r="I1017" t="n">
+        <v>240000</v>
+      </c>
+      <c r="J1017" t="inlineStr">
+        <is>
+          <t>efectivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="1018">
+      <c r="A1018" s="3" t="n">
+        <v>46184</v>
+      </c>
+      <c r="B1018" t="inlineStr">
+        <is>
+          <t>Ana Milena Juan Davit</t>
+        </is>
+      </c>
+      <c r="C1018" t="inlineStr">
+        <is>
+          <t>Bajaj UPY 65H</t>
+        </is>
+      </c>
+      <c r="D1018" t="inlineStr">
+        <is>
+          <t>UPY65H</t>
+        </is>
+      </c>
+      <c r="H1018" t="n">
+        <v>240000</v>
+      </c>
+      <c r="I1018" t="n">
+        <v>240000</v>
+      </c>
+      <c r="J1018" t="inlineStr">
+        <is>
+          <t>efectivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="1019">
+      <c r="A1019" s="3" t="n">
+        <v>46191</v>
+      </c>
+      <c r="B1019" t="inlineStr">
+        <is>
+          <t>Ana Milena Juan Davit</t>
+        </is>
+      </c>
+      <c r="C1019" t="inlineStr">
+        <is>
+          <t>Bajaj UPY 65H</t>
+        </is>
+      </c>
+      <c r="D1019" t="inlineStr">
+        <is>
+          <t>UPY65H</t>
+        </is>
+      </c>
+      <c r="H1019" t="n">
+        <v>240000</v>
+      </c>
+      <c r="I1019" t="n">
+        <v>240000</v>
+      </c>
+      <c r="J1019" t="inlineStr">
+        <is>
+          <t>efectivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="1020">
+      <c r="A1020" s="3" t="n">
+        <v>46198</v>
+      </c>
+      <c r="B1020" t="inlineStr">
+        <is>
+          <t>Ana Milena Juan Davit</t>
+        </is>
+      </c>
+      <c r="C1020" t="inlineStr">
+        <is>
+          <t>Bajaj UPY 65H</t>
+        </is>
+      </c>
+      <c r="D1020" t="inlineStr">
+        <is>
+          <t>UPY65H</t>
+        </is>
+      </c>
+      <c r="H1020" t="n">
+        <v>240000</v>
+      </c>
+      <c r="I1020" t="n">
+        <v>240000</v>
+      </c>
+      <c r="J1020" t="inlineStr">
+        <is>
+          <t>efectivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="1021">
+      <c r="A1021" s="3" t="n">
+        <v>46205</v>
+      </c>
+      <c r="B1021" t="inlineStr">
+        <is>
+          <t>Ana Milena Juan Davit</t>
+        </is>
+      </c>
+      <c r="C1021" t="inlineStr">
+        <is>
+          <t>Bajaj UPY 65H</t>
+        </is>
+      </c>
+      <c r="D1021" t="inlineStr">
+        <is>
+          <t>UPY65H</t>
+        </is>
+      </c>
+      <c r="H1021" t="n">
+        <v>240000</v>
+      </c>
+      <c r="I1021" t="n">
+        <v>240000</v>
+      </c>
+      <c r="J1021" t="inlineStr">
+        <is>
+          <t>efectivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="1022">
+      <c r="A1022" s="3" t="n">
+        <v>46212</v>
+      </c>
+      <c r="B1022" t="inlineStr">
+        <is>
+          <t>Ana Milena Juan Davit</t>
+        </is>
+      </c>
+      <c r="C1022" t="inlineStr">
+        <is>
+          <t>Bajaj UPY 65H</t>
+        </is>
+      </c>
+      <c r="D1022" t="inlineStr">
+        <is>
+          <t>UPY65H</t>
+        </is>
+      </c>
+      <c r="H1022" t="n">
+        <v>240000</v>
+      </c>
+      <c r="I1022" t="n">
+        <v>240000</v>
+      </c>
+      <c r="J1022" t="inlineStr">
+        <is>
+          <t>efectivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="1023">
+      <c r="A1023" s="3" t="n">
+        <v>46219</v>
+      </c>
+      <c r="B1023" t="inlineStr">
+        <is>
+          <t>Ana Milena Juan Davit</t>
+        </is>
+      </c>
+      <c r="C1023" t="inlineStr">
+        <is>
+          <t>Bajaj UPY 65H</t>
+        </is>
+      </c>
+      <c r="D1023" t="inlineStr">
+        <is>
+          <t>UPY65H</t>
+        </is>
+      </c>
+      <c r="H1023" t="n">
+        <v>240000</v>
+      </c>
+      <c r="I1023" t="n">
+        <v>240000</v>
+      </c>
+      <c r="J1023" t="inlineStr">
+        <is>
+          <t>efectivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="1024">
+      <c r="A1024" s="3" t="n">
+        <v>46027</v>
+      </c>
+      <c r="B1024" t="inlineStr">
+        <is>
+          <t>Sr Luis</t>
+        </is>
+      </c>
+      <c r="C1024" t="inlineStr">
+        <is>
+          <t>Bajaj UYZ 32H</t>
+        </is>
+      </c>
+      <c r="D1024" t="inlineStr">
+        <is>
+          <t>UYZ32H</t>
+        </is>
+      </c>
+      <c r="H1024" t="n">
+        <v>240000</v>
+      </c>
+      <c r="I1024" t="n">
+        <v>240000</v>
+      </c>
+      <c r="J1024" t="inlineStr">
+        <is>
+          <t>efectivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="1025">
+      <c r="A1025" s="3" t="n">
+        <v>46035</v>
+      </c>
+      <c r="B1025" t="inlineStr">
+        <is>
+          <t>Sr Luis</t>
+        </is>
+      </c>
+      <c r="C1025" t="inlineStr">
+        <is>
+          <t>Bajaj UYZ 32H</t>
+        </is>
+      </c>
+      <c r="D1025" t="inlineStr">
+        <is>
+          <t>UYZ32H</t>
+        </is>
+      </c>
+      <c r="H1025" t="n">
+        <v>240000</v>
+      </c>
+      <c r="I1025" t="n">
+        <v>240000</v>
+      </c>
+      <c r="J1025" t="inlineStr">
+        <is>
+          <t>efectivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="1026">
+      <c r="A1026" s="3" t="n">
+        <v>46043</v>
+      </c>
+      <c r="B1026" t="inlineStr">
+        <is>
+          <t>Sr Luis</t>
+        </is>
+      </c>
+      <c r="C1026" t="inlineStr">
+        <is>
+          <t>Bajaj UYZ 32H</t>
+        </is>
+      </c>
+      <c r="D1026" t="inlineStr">
+        <is>
+          <t>UYZ32H</t>
+        </is>
+      </c>
+      <c r="H1026" t="n">
+        <v>240000</v>
+      </c>
+      <c r="I1026" t="n">
+        <v>240000</v>
+      </c>
+      <c r="J1026" t="inlineStr">
+        <is>
+          <t>efectivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="1027">
+      <c r="A1027" s="3" t="n">
+        <v>46051</v>
+      </c>
+      <c r="B1027" t="inlineStr">
+        <is>
+          <t>Sr Luis</t>
+        </is>
+      </c>
+      <c r="C1027" t="inlineStr">
+        <is>
+          <t>Bajaj UYZ 32H</t>
+        </is>
+      </c>
+      <c r="D1027" t="inlineStr">
+        <is>
+          <t>UYZ32H</t>
+        </is>
+      </c>
+      <c r="H1027" t="n">
+        <v>240000</v>
+      </c>
+      <c r="I1027" t="n">
+        <v>240000</v>
+      </c>
+      <c r="J1027" t="inlineStr">
+        <is>
+          <t>efectivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="1028">
+      <c r="A1028" s="3" t="n">
+        <v>46059</v>
+      </c>
+      <c r="B1028" t="inlineStr">
+        <is>
+          <t>Sr Luis</t>
+        </is>
+      </c>
+      <c r="C1028" t="inlineStr">
+        <is>
+          <t>Bajaj UYZ 32H</t>
+        </is>
+      </c>
+      <c r="D1028" t="inlineStr">
+        <is>
+          <t>UYZ32H</t>
+        </is>
+      </c>
+      <c r="H1028" t="n">
+        <v>240000</v>
+      </c>
+      <c r="I1028" t="n">
+        <v>240000</v>
+      </c>
+      <c r="J1028" t="inlineStr">
+        <is>
+          <t>efectivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="1029">
+      <c r="A1029" s="3" t="n">
+        <v>46067</v>
+      </c>
+      <c r="B1029" t="inlineStr">
+        <is>
+          <t>Sr Luis</t>
+        </is>
+      </c>
+      <c r="C1029" t="inlineStr">
+        <is>
+          <t>Bajaj UYZ 32H</t>
+        </is>
+      </c>
+      <c r="D1029" t="inlineStr">
+        <is>
+          <t>UYZ32H</t>
+        </is>
+      </c>
+      <c r="H1029" t="n">
+        <v>240000</v>
+      </c>
+      <c r="I1029" t="n">
+        <v>240000</v>
+      </c>
+      <c r="J1029" t="inlineStr">
+        <is>
+          <t>efectivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="1030">
+      <c r="A1030" s="3" t="n">
+        <v>46075</v>
+      </c>
+      <c r="B1030" t="inlineStr">
+        <is>
+          <t>Sr Luis</t>
+        </is>
+      </c>
+      <c r="C1030" t="inlineStr">
+        <is>
+          <t>Bajaj UYZ 32H</t>
+        </is>
+      </c>
+      <c r="D1030" t="inlineStr">
+        <is>
+          <t>UYZ32H</t>
+        </is>
+      </c>
+      <c r="H1030" t="n">
+        <v>240000</v>
+      </c>
+      <c r="I1030" t="n">
+        <v>240000</v>
+      </c>
+      <c r="J1030" t="inlineStr">
+        <is>
+          <t>efectivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="1031">
+      <c r="A1031" s="3" t="n">
+        <v>46083</v>
+      </c>
+      <c r="B1031" t="inlineStr">
+        <is>
+          <t>Sr Luis</t>
+        </is>
+      </c>
+      <c r="C1031" t="inlineStr">
+        <is>
+          <t>Bajaj UYZ 32H</t>
+        </is>
+      </c>
+      <c r="D1031" t="inlineStr">
+        <is>
+          <t>UYZ32H</t>
+        </is>
+      </c>
+      <c r="H1031" t="n">
+        <v>240000</v>
+      </c>
+      <c r="I1031" t="n">
+        <v>240000</v>
+      </c>
+      <c r="J1031" t="inlineStr">
+        <is>
+          <t>efectivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="1032">
+      <c r="A1032" s="3" t="n">
+        <v>46091</v>
+      </c>
+      <c r="B1032" t="inlineStr">
+        <is>
+          <t>Sr Luis</t>
+        </is>
+      </c>
+      <c r="C1032" t="inlineStr">
+        <is>
+          <t>Bajaj UYZ 32H</t>
+        </is>
+      </c>
+      <c r="D1032" t="inlineStr">
+        <is>
+          <t>UYZ32H</t>
+        </is>
+      </c>
+      <c r="H1032" t="n">
+        <v>240000</v>
+      </c>
+      <c r="I1032" t="n">
+        <v>240000</v>
+      </c>
+      <c r="J1032" t="inlineStr">
+        <is>
+          <t>efectivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="1033">
+      <c r="A1033" s="3" t="n">
+        <v>46099</v>
+      </c>
+      <c r="B1033" t="inlineStr">
+        <is>
+          <t>Sr Luis</t>
+        </is>
+      </c>
+      <c r="C1033" t="inlineStr">
+        <is>
+          <t>Bajaj UYZ 32H</t>
+        </is>
+      </c>
+      <c r="D1033" t="inlineStr">
+        <is>
+          <t>UYZ32H</t>
+        </is>
+      </c>
+      <c r="H1033" t="n">
+        <v>240000</v>
+      </c>
+      <c r="I1033" t="n">
+        <v>240000</v>
+      </c>
+      <c r="J1033" t="inlineStr">
+        <is>
+          <t>efectivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="1034">
+      <c r="A1034" s="3" t="n">
+        <v>46107</v>
+      </c>
+      <c r="B1034" t="inlineStr">
+        <is>
+          <t>Sr Luis</t>
+        </is>
+      </c>
+      <c r="C1034" t="inlineStr">
+        <is>
+          <t>Bajaj UYZ 32H</t>
+        </is>
+      </c>
+      <c r="D1034" t="inlineStr">
+        <is>
+          <t>UYZ32H</t>
+        </is>
+      </c>
+      <c r="H1034" t="n">
+        <v>240000</v>
+      </c>
+      <c r="I1034" t="n">
+        <v>240000</v>
+      </c>
+      <c r="J1034" t="inlineStr">
+        <is>
+          <t>efectivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="1035">
+      <c r="A1035" s="3" t="n">
+        <v>46115</v>
+      </c>
+      <c r="B1035" t="inlineStr">
+        <is>
+          <t>Sr Luis</t>
+        </is>
+      </c>
+      <c r="C1035" t="inlineStr">
+        <is>
+          <t>Bajaj UYZ 32H</t>
+        </is>
+      </c>
+      <c r="D1035" t="inlineStr">
+        <is>
+          <t>UYZ32H</t>
+        </is>
+      </c>
+      <c r="H1035" t="n">
+        <v>240000</v>
+      </c>
+      <c r="I1035" t="n">
+        <v>240000</v>
+      </c>
+      <c r="J1035" t="inlineStr">
+        <is>
+          <t>efectivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="1036">
+      <c r="A1036" s="3" t="n">
+        <v>46123</v>
+      </c>
+      <c r="B1036" t="inlineStr">
+        <is>
+          <t>Sr Luis</t>
+        </is>
+      </c>
+      <c r="C1036" t="inlineStr">
+        <is>
+          <t>Bajaj UYZ 32H</t>
+        </is>
+      </c>
+      <c r="D1036" t="inlineStr">
+        <is>
+          <t>UYZ32H</t>
+        </is>
+      </c>
+      <c r="H1036" t="n">
+        <v>240000</v>
+      </c>
+      <c r="I1036" t="n">
+        <v>240000</v>
+      </c>
+      <c r="J1036" t="inlineStr">
+        <is>
+          <t>efectivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="1037">
+      <c r="A1037" s="3" t="n">
+        <v>46131</v>
+      </c>
+      <c r="B1037" t="inlineStr">
+        <is>
+          <t>Sr Luis</t>
+        </is>
+      </c>
+      <c r="C1037" t="inlineStr">
+        <is>
+          <t>Bajaj UYZ 32H</t>
+        </is>
+      </c>
+      <c r="D1037" t="inlineStr">
+        <is>
+          <t>UYZ32H</t>
+        </is>
+      </c>
+      <c r="H1037" t="n">
+        <v>240000</v>
+      </c>
+      <c r="I1037" t="n">
+        <v>240000</v>
+      </c>
+      <c r="J1037" t="inlineStr">
+        <is>
+          <t>efectivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="1038">
+      <c r="A1038" s="3" t="n">
+        <v>46065</v>
+      </c>
+      <c r="B1038" t="inlineStr">
+        <is>
+          <t>Manuel Alga</t>
+        </is>
+      </c>
+      <c r="C1038" t="inlineStr">
+        <is>
+          <t>Bajaj UYZ 39H</t>
+        </is>
+      </c>
+      <c r="D1038" t="inlineStr">
+        <is>
+          <t>UYZ39H</t>
+        </is>
+      </c>
+      <c r="H1038" t="n">
+        <v>240000</v>
+      </c>
+      <c r="I1038" t="n">
+        <v>240000</v>
+      </c>
+      <c r="J1038" t="inlineStr">
+        <is>
+          <t>efectivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="1039">
+      <c r="A1039" s="3" t="n">
+        <v>46077</v>
+      </c>
+      <c r="B1039" t="inlineStr">
+        <is>
+          <t>Manuel Alga</t>
+        </is>
+      </c>
+      <c r="C1039" t="inlineStr">
+        <is>
+          <t>Bajaj UYZ 39H</t>
+        </is>
+      </c>
+      <c r="D1039" t="inlineStr">
+        <is>
+          <t>UYZ39H</t>
+        </is>
+      </c>
+      <c r="H1039" t="n">
+        <v>240000</v>
+      </c>
+      <c r="I1039" t="n">
+        <v>240000</v>
+      </c>
+      <c r="J1039" t="inlineStr">
+        <is>
+          <t>efectivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="1040">
+      <c r="A1040" s="3" t="n">
+        <v>46086</v>
+      </c>
+      <c r="B1040" t="inlineStr">
+        <is>
+          <t>Manuel Alga</t>
+        </is>
+      </c>
+      <c r="C1040" t="inlineStr">
+        <is>
+          <t>Bajaj UYZ 39H</t>
+        </is>
+      </c>
+      <c r="D1040" t="inlineStr">
+        <is>
+          <t>UYZ39H</t>
+        </is>
+      </c>
+      <c r="H1040" t="n">
+        <v>240000</v>
+      </c>
+      <c r="I1040" t="n">
+        <v>240000</v>
+      </c>
+      <c r="J1040" t="inlineStr">
+        <is>
+          <t>efectivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="1041">
+      <c r="A1041" s="3" t="n">
+        <v>46090</v>
+      </c>
+      <c r="B1041" t="inlineStr">
+        <is>
+          <t>Manuel Alga</t>
+        </is>
+      </c>
+      <c r="C1041" t="inlineStr">
+        <is>
+          <t>Bajaj UYZ 39H</t>
+        </is>
+      </c>
+      <c r="D1041" t="inlineStr">
+        <is>
+          <t>UYZ39H</t>
+        </is>
+      </c>
+      <c r="H1041" t="n">
+        <v>240000</v>
+      </c>
+      <c r="I1041" t="n">
+        <v>240000</v>
+      </c>
+      <c r="J1041" t="inlineStr">
+        <is>
+          <t>efectivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="1042">
+      <c r="A1042" s="3" t="n">
+        <v>46097</v>
+      </c>
+      <c r="B1042" t="inlineStr">
+        <is>
+          <t>Manuel Alga</t>
+        </is>
+      </c>
+      <c r="C1042" t="inlineStr">
+        <is>
+          <t>Bajaj UYZ 39H</t>
+        </is>
+      </c>
+      <c r="D1042" t="inlineStr">
+        <is>
+          <t>UYZ39H</t>
+        </is>
+      </c>
+      <c r="H1042" t="n">
+        <v>240000</v>
+      </c>
+      <c r="I1042" t="n">
+        <v>240000</v>
+      </c>
+      <c r="J1042" t="inlineStr">
+        <is>
+          <t>efectivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="1043">
+      <c r="A1043" s="3" t="n">
+        <v>46106</v>
+      </c>
+      <c r="B1043" t="inlineStr">
+        <is>
+          <t>Manuel Alga</t>
+        </is>
+      </c>
+      <c r="C1043" t="inlineStr">
+        <is>
+          <t>Bajaj UYZ 39H</t>
+        </is>
+      </c>
+      <c r="D1043" t="inlineStr">
+        <is>
+          <t>UYZ39H</t>
+        </is>
+      </c>
+      <c r="H1043" t="n">
+        <v>240000</v>
+      </c>
+      <c r="I1043" t="n">
+        <v>240000</v>
+      </c>
+      <c r="J1043" t="inlineStr">
+        <is>
+          <t>efectivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="1044">
+      <c r="A1044" s="3" t="n">
+        <v>46118</v>
+      </c>
+      <c r="B1044" t="inlineStr">
+        <is>
+          <t>Manuel Alga</t>
+        </is>
+      </c>
+      <c r="C1044" t="inlineStr">
+        <is>
+          <t>Bajaj UYZ 39H</t>
+        </is>
+      </c>
+      <c r="D1044" t="inlineStr">
+        <is>
+          <t>UYZ39H</t>
+        </is>
+      </c>
+      <c r="H1044" t="n">
+        <v>240000</v>
+      </c>
+      <c r="I1044" t="n">
+        <v>240000</v>
+      </c>
+      <c r="J1044" t="inlineStr">
+        <is>
+          <t>efectivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="1045">
+      <c r="A1045" s="3" t="n">
+        <v>46126</v>
+      </c>
+      <c r="B1045" t="inlineStr">
+        <is>
+          <t>Manuel Alga</t>
+        </is>
+      </c>
+      <c r="C1045" t="inlineStr">
+        <is>
+          <t>Bajaj UYZ 39H</t>
+        </is>
+      </c>
+      <c r="D1045" t="inlineStr">
+        <is>
+          <t>UYZ39H</t>
+        </is>
+      </c>
+      <c r="H1045" t="n">
+        <v>240000</v>
+      </c>
+      <c r="I1045" t="n">
+        <v>240000</v>
+      </c>
+      <c r="J1045" t="inlineStr">
+        <is>
+          <t>efectivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="1046">
+      <c r="A1046" s="3" t="n">
+        <v>46137</v>
+      </c>
+      <c r="B1046" t="inlineStr">
+        <is>
+          <t>Manuel Alga</t>
+        </is>
+      </c>
+      <c r="C1046" t="inlineStr">
+        <is>
+          <t>Bajaj UYZ 39H</t>
+        </is>
+      </c>
+      <c r="D1046" t="inlineStr">
+        <is>
+          <t>UYZ39H</t>
+        </is>
+      </c>
+      <c r="H1046" t="n">
+        <v>240000</v>
+      </c>
+      <c r="I1046" t="n">
+        <v>240000</v>
+      </c>
+      <c r="J1046" t="inlineStr">
+        <is>
+          <t>efectivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="1047">
+      <c r="A1047" s="3" t="n">
+        <v>46146</v>
+      </c>
+      <c r="B1047" t="inlineStr">
+        <is>
+          <t>Manuel Alga</t>
+        </is>
+      </c>
+      <c r="C1047" t="inlineStr">
+        <is>
+          <t>Bajaj UYZ 39H</t>
+        </is>
+      </c>
+      <c r="D1047" t="inlineStr">
+        <is>
+          <t>UYZ39H</t>
+        </is>
+      </c>
+      <c r="H1047" t="n">
+        <v>240000</v>
+      </c>
+      <c r="I1047" t="n">
+        <v>240000</v>
+      </c>
+      <c r="J1047" t="inlineStr">
+        <is>
+          <t>efectivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="1048">
+      <c r="A1048" s="3" t="n">
+        <v>46161</v>
+      </c>
+      <c r="B1048" t="inlineStr">
+        <is>
+          <t>Manuel Alga</t>
+        </is>
+      </c>
+      <c r="C1048" t="inlineStr">
+        <is>
+          <t>Bajaj UYZ 39H</t>
+        </is>
+      </c>
+      <c r="D1048" t="inlineStr">
+        <is>
+          <t>UYZ39H</t>
+        </is>
+      </c>
+      <c r="H1048" t="n">
+        <v>240000</v>
+      </c>
+      <c r="I1048" t="n">
+        <v>240000</v>
+      </c>
+      <c r="J1048" t="inlineStr">
+        <is>
+          <t>efectivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="1049">
+      <c r="A1049" s="3" t="n">
+        <v>46171</v>
+      </c>
+      <c r="B1049" t="inlineStr">
+        <is>
+          <t>Manuel Alga</t>
+        </is>
+      </c>
+      <c r="C1049" t="inlineStr">
+        <is>
+          <t>Bajaj UYZ 39H</t>
+        </is>
+      </c>
+      <c r="D1049" t="inlineStr">
+        <is>
+          <t>UYZ39H</t>
+        </is>
+      </c>
+      <c r="H1049" t="n">
+        <v>240000</v>
+      </c>
+      <c r="I1049" t="n">
+        <v>240000</v>
+      </c>
+      <c r="J1049" t="inlineStr">
+        <is>
+          <t>efectivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="1050">
+      <c r="A1050" s="3" t="n">
+        <v>46181</v>
+      </c>
+      <c r="B1050" t="inlineStr">
+        <is>
+          <t>Manuel Alga</t>
+        </is>
+      </c>
+      <c r="C1050" t="inlineStr">
+        <is>
+          <t>Bajaj UYZ 39H</t>
+        </is>
+      </c>
+      <c r="D1050" t="inlineStr">
+        <is>
+          <t>UYZ39H</t>
+        </is>
+      </c>
+      <c r="H1050" t="n">
+        <v>240000</v>
+      </c>
+      <c r="I1050" t="n">
+        <v>240000</v>
+      </c>
+      <c r="J1050" t="inlineStr">
+        <is>
+          <t>efectivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="1051">
+      <c r="A1051" s="3" t="n">
+        <v>46190</v>
+      </c>
+      <c r="B1051" t="inlineStr">
+        <is>
+          <t>Manuel Alga</t>
+        </is>
+      </c>
+      <c r="C1051" t="inlineStr">
+        <is>
+          <t>Bajaj UYZ 39H</t>
+        </is>
+      </c>
+      <c r="D1051" t="inlineStr">
+        <is>
+          <t>UYZ39H</t>
+        </is>
+      </c>
+      <c r="H1051" t="n">
+        <v>240000</v>
+      </c>
+      <c r="I1051" t="n">
+        <v>240000</v>
+      </c>
+      <c r="J1051" t="inlineStr">
+        <is>
+          <t>efectivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="1052">
+      <c r="A1052" s="3" t="n">
+        <v>46198</v>
+      </c>
+      <c r="B1052" t="inlineStr">
+        <is>
+          <t>Manuel Alga</t>
+        </is>
+      </c>
+      <c r="C1052" t="inlineStr">
+        <is>
+          <t>Bajaj UYZ 39H</t>
+        </is>
+      </c>
+      <c r="D1052" t="inlineStr">
+        <is>
+          <t>UYZ39H</t>
+        </is>
+      </c>
+      <c r="H1052" t="n">
+        <v>240000</v>
+      </c>
+      <c r="I1052" t="n">
+        <v>240000</v>
+      </c>
+      <c r="J1052" t="inlineStr">
+        <is>
+          <t>efectivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="1053">
+      <c r="A1053" s="3" t="n">
+        <v>46208</v>
+      </c>
+      <c r="B1053" t="inlineStr">
+        <is>
+          <t>Manuel Alga</t>
+        </is>
+      </c>
+      <c r="C1053" t="inlineStr">
+        <is>
+          <t>Bajaj UYZ 39H</t>
+        </is>
+      </c>
+      <c r="D1053" t="inlineStr">
+        <is>
+          <t>UYZ39H</t>
+        </is>
+      </c>
+      <c r="H1053" t="n">
+        <v>240000</v>
+      </c>
+      <c r="I1053" t="n">
+        <v>240000</v>
+      </c>
+      <c r="J1053" t="inlineStr">
+        <is>
+          <t>efectivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="1054">
+      <c r="A1054" s="3" t="n">
+        <v>46211</v>
+      </c>
+      <c r="B1054" t="inlineStr">
+        <is>
+          <t>Manuel Alga</t>
+        </is>
+      </c>
+      <c r="C1054" t="inlineStr">
+        <is>
+          <t>Bajaj UYZ 39H</t>
+        </is>
+      </c>
+      <c r="D1054" t="inlineStr">
+        <is>
+          <t>UYZ39H</t>
+        </is>
+      </c>
+      <c r="H1054" t="n">
+        <v>240000</v>
+      </c>
+      <c r="I1054" t="n">
+        <v>240000</v>
+      </c>
+      <c r="J1054" t="inlineStr">
+        <is>
+          <t>efectivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="1055">
+      <c r="A1055" s="3" t="n">
+        <v>46224</v>
+      </c>
+      <c r="B1055" t="inlineStr">
+        <is>
+          <t>Manuel Alga</t>
+        </is>
+      </c>
+      <c r="C1055" t="inlineStr">
+        <is>
+          <t>Bajaj UYZ 39H</t>
+        </is>
+      </c>
+      <c r="D1055" t="inlineStr">
+        <is>
+          <t>UYZ39H</t>
+        </is>
+      </c>
+      <c r="H1055" t="n">
+        <v>240000</v>
+      </c>
+      <c r="I1055" t="n">
+        <v>240000</v>
+      </c>
+      <c r="J1055" t="inlineStr">
+        <is>
+          <t>efectivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="1056">
+      <c r="A1056" s="3" t="n">
+        <v>46069</v>
+      </c>
+      <c r="B1056" t="inlineStr">
+        <is>
+          <t>Jorge Estrada</t>
+        </is>
+      </c>
+      <c r="C1056" t="inlineStr">
+        <is>
+          <t>Bajaj BJH 66I</t>
+        </is>
+      </c>
+      <c r="D1056" t="inlineStr">
+        <is>
+          <t>BJH66I</t>
+        </is>
+      </c>
+      <c r="H1056" t="n">
+        <v>240000</v>
+      </c>
+      <c r="I1056" t="n">
+        <v>240000</v>
+      </c>
+      <c r="J1056" t="inlineStr">
+        <is>
+          <t>efectivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="1057">
+      <c r="A1057" s="3" t="n">
+        <v>46077</v>
+      </c>
+      <c r="B1057" t="inlineStr">
+        <is>
+          <t>Jorge Estrada</t>
+        </is>
+      </c>
+      <c r="C1057" t="inlineStr">
+        <is>
+          <t>Bajaj BJH 66I</t>
+        </is>
+      </c>
+      <c r="D1057" t="inlineStr">
+        <is>
+          <t>BJH66I</t>
+        </is>
+      </c>
+      <c r="H1057" t="n">
+        <v>240000</v>
+      </c>
+      <c r="I1057" t="n">
+        <v>240000</v>
+      </c>
+      <c r="J1057" t="inlineStr">
+        <is>
+          <t>efectivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="1058">
+      <c r="A1058" s="3" t="n">
+        <v>46082</v>
+      </c>
+      <c r="B1058" t="inlineStr">
+        <is>
+          <t>Jorge Estrada</t>
+        </is>
+      </c>
+      <c r="C1058" t="inlineStr">
+        <is>
+          <t>Bajaj BJH 66I</t>
+        </is>
+      </c>
+      <c r="D1058" t="inlineStr">
+        <is>
+          <t>BJH66I</t>
+        </is>
+      </c>
+      <c r="H1058" t="n">
+        <v>240000</v>
+      </c>
+      <c r="I1058" t="n">
+        <v>240000</v>
+      </c>
+      <c r="J1058" t="inlineStr">
+        <is>
+          <t>efectivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="1059">
+      <c r="A1059" s="3" t="n">
+        <v>46090</v>
+      </c>
+      <c r="B1059" t="inlineStr">
+        <is>
+          <t>Jorge Estrada</t>
+        </is>
+      </c>
+      <c r="C1059" t="inlineStr">
+        <is>
+          <t>Bajaj BJH 66I</t>
+        </is>
+      </c>
+      <c r="D1059" t="inlineStr">
+        <is>
+          <t>BJH66I</t>
+        </is>
+      </c>
+      <c r="H1059" t="n">
+        <v>240000</v>
+      </c>
+      <c r="I1059" t="n">
+        <v>240000</v>
+      </c>
+      <c r="J1059" t="inlineStr">
+        <is>
+          <t>efectivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="1060">
+      <c r="A1060" s="3" t="n">
+        <v>46098</v>
+      </c>
+      <c r="B1060" t="inlineStr">
+        <is>
+          <t>Jorge Estrada</t>
+        </is>
+      </c>
+      <c r="C1060" t="inlineStr">
+        <is>
+          <t>Bajaj BJH 66I</t>
+        </is>
+      </c>
+      <c r="D1060" t="inlineStr">
+        <is>
+          <t>BJH66I</t>
+        </is>
+      </c>
+      <c r="H1060" t="n">
+        <v>240000</v>
+      </c>
+      <c r="I1060" t="n">
+        <v>240000</v>
+      </c>
+      <c r="J1060" t="inlineStr">
+        <is>
+          <t>efectivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="1061">
+      <c r="A1061" s="3" t="n">
+        <v>46105</v>
+      </c>
+      <c r="B1061" t="inlineStr">
+        <is>
+          <t>Jorge Estrada</t>
+        </is>
+      </c>
+      <c r="C1061" t="inlineStr">
+        <is>
+          <t>Bajaj BJH 66I</t>
+        </is>
+      </c>
+      <c r="D1061" t="inlineStr">
+        <is>
+          <t>BJH66I</t>
+        </is>
+      </c>
+      <c r="H1061" t="n">
+        <v>240000</v>
+      </c>
+      <c r="I1061" t="n">
+        <v>240000</v>
+      </c>
+      <c r="J1061" t="inlineStr">
+        <is>
+          <t>efectivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="1062">
+      <c r="A1062" s="3" t="n">
+        <v>46115</v>
+      </c>
+      <c r="B1062" t="inlineStr">
+        <is>
+          <t>Jorge Estrada</t>
+        </is>
+      </c>
+      <c r="C1062" t="inlineStr">
+        <is>
+          <t>Bajaj BJH 66I</t>
+        </is>
+      </c>
+      <c r="D1062" t="inlineStr">
+        <is>
+          <t>BJH66I</t>
+        </is>
+      </c>
+      <c r="H1062" t="n">
+        <v>240000</v>
+      </c>
+      <c r="I1062" t="n">
+        <v>240000</v>
+      </c>
+      <c r="J1062" t="inlineStr">
+        <is>
+          <t>efectivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="1063">
+      <c r="A1063" s="3" t="n">
+        <v>46126</v>
+      </c>
+      <c r="B1063" t="inlineStr">
+        <is>
+          <t>Jorge Estrada</t>
+        </is>
+      </c>
+      <c r="C1063" t="inlineStr">
+        <is>
+          <t>Bajaj BJH 66I</t>
+        </is>
+      </c>
+      <c r="D1063" t="inlineStr">
+        <is>
+          <t>BJH66I</t>
+        </is>
+      </c>
+      <c r="H1063" t="n">
+        <v>240000</v>
+      </c>
+      <c r="I1063" t="n">
+        <v>240000</v>
+      </c>
+      <c r="J1063" t="inlineStr">
+        <is>
+          <t>efectivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="1064">
+      <c r="A1064" s="3" t="n">
+        <v>46133</v>
+      </c>
+      <c r="B1064" t="inlineStr">
+        <is>
+          <t>Jorge Estrada</t>
+        </is>
+      </c>
+      <c r="C1064" t="inlineStr">
+        <is>
+          <t>Bajaj BJH 66I</t>
+        </is>
+      </c>
+      <c r="D1064" t="inlineStr">
+        <is>
+          <t>BJH66I</t>
+        </is>
+      </c>
+      <c r="H1064" t="n">
+        <v>240000</v>
+      </c>
+      <c r="I1064" t="n">
+        <v>240000</v>
+      </c>
+      <c r="J1064" t="inlineStr">
+        <is>
+          <t>efectivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="1065">
+      <c r="A1065" s="3" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B1065" t="inlineStr">
+        <is>
+          <t>Jorge Estrada</t>
+        </is>
+      </c>
+      <c r="C1065" t="inlineStr">
+        <is>
+          <t>Bajaj BJH 66I</t>
+        </is>
+      </c>
+      <c r="D1065" t="inlineStr">
+        <is>
+          <t>BJH66I</t>
+        </is>
+      </c>
+      <c r="H1065" t="n">
+        <v>240000</v>
+      </c>
+      <c r="I1065" t="n">
+        <v>240000</v>
+      </c>
+      <c r="J1065" t="inlineStr">
+        <is>
+          <t>efectivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="1066">
+      <c r="A1066" s="3" t="n">
+        <v>46182</v>
+      </c>
+      <c r="B1066" t="inlineStr">
+        <is>
+          <t>Jorge Estrada</t>
+        </is>
+      </c>
+      <c r="C1066" t="inlineStr">
+        <is>
+          <t>Bajaj BJH 66I</t>
+        </is>
+      </c>
+      <c r="D1066" t="inlineStr">
+        <is>
+          <t>BJH66I</t>
+        </is>
+      </c>
+      <c r="H1066" t="n">
+        <v>240000</v>
+      </c>
+      <c r="I1066" t="n">
+        <v>240000</v>
+      </c>
+      <c r="J1066" t="inlineStr">
+        <is>
+          <t>efectivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="1067">
+      <c r="A1067" s="3" t="n">
+        <v>46189</v>
+      </c>
+      <c r="B1067" t="inlineStr">
+        <is>
+          <t>Jorge Estrada</t>
+        </is>
+      </c>
+      <c r="C1067" t="inlineStr">
+        <is>
+          <t>Bajaj BJH 66I</t>
+        </is>
+      </c>
+      <c r="D1067" t="inlineStr">
+        <is>
+          <t>BJH66I</t>
+        </is>
+      </c>
+      <c r="H1067" t="n">
+        <v>240000</v>
+      </c>
+      <c r="I1067" t="n">
+        <v>240000</v>
+      </c>
+      <c r="J1067" t="inlineStr">
+        <is>
+          <t>efectivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="1068">
+      <c r="A1068" s="3" t="n">
+        <v>46197</v>
+      </c>
+      <c r="B1068" t="inlineStr">
+        <is>
+          <t>Jorge Estrada</t>
+        </is>
+      </c>
+      <c r="C1068" t="inlineStr">
+        <is>
+          <t>Bajaj BJH 66I</t>
+        </is>
+      </c>
+      <c r="D1068" t="inlineStr">
+        <is>
+          <t>BJH66I</t>
+        </is>
+      </c>
+      <c r="H1068" t="n">
+        <v>240000</v>
+      </c>
+      <c r="I1068" t="n">
+        <v>240000</v>
+      </c>
+      <c r="J1068" t="inlineStr">
+        <is>
+          <t>efectivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="1069">
+      <c r="A1069" s="3" t="n">
+        <v>46204</v>
+      </c>
+      <c r="B1069" t="inlineStr">
+        <is>
+          <t>Jorge Estrada</t>
+        </is>
+      </c>
+      <c r="C1069" t="inlineStr">
+        <is>
+          <t>Bajaj BJH 66I</t>
+        </is>
+      </c>
+      <c r="D1069" t="inlineStr">
+        <is>
+          <t>BJH66I</t>
+        </is>
+      </c>
+      <c r="H1069" t="n">
+        <v>240000</v>
+      </c>
+      <c r="I1069" t="n">
+        <v>240000</v>
+      </c>
+      <c r="J1069" t="inlineStr">
+        <is>
+          <t>efectivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="1070">
+      <c r="A1070" s="3" t="n">
+        <v>46213</v>
+      </c>
+      <c r="B1070" t="inlineStr">
+        <is>
+          <t>Jorge Estrada</t>
+        </is>
+      </c>
+      <c r="C1070" t="inlineStr">
+        <is>
+          <t>Bajaj BJH 66I</t>
+        </is>
+      </c>
+      <c r="D1070" t="inlineStr">
+        <is>
+          <t>BJH66I</t>
+        </is>
+      </c>
+      <c r="H1070" t="n">
+        <v>240000</v>
+      </c>
+      <c r="I1070" t="n">
+        <v>240000</v>
+      </c>
+      <c r="J1070" t="inlineStr">
+        <is>
+          <t>efectivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="1071">
+      <c r="A1071" s="3" t="n">
+        <v>46224</v>
+      </c>
+      <c r="B1071" t="inlineStr">
+        <is>
+          <t>Jorge Estrada</t>
+        </is>
+      </c>
+      <c r="C1071" t="inlineStr">
+        <is>
+          <t>Bajaj BJH 66I</t>
+        </is>
+      </c>
+      <c r="D1071" t="inlineStr">
+        <is>
+          <t>BJH66I</t>
+        </is>
+      </c>
+      <c r="H1071" t="n">
+        <v>240000</v>
+      </c>
+      <c r="I1071" t="n">
+        <v>240000</v>
+      </c>
+      <c r="J1071" t="inlineStr">
+        <is>
+          <t>efectivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="1072">
+      <c r="A1072" s="3" t="n">
+        <v>46086</v>
+      </c>
+      <c r="B1072" t="inlineStr">
+        <is>
+          <t>Donita Juan Camilo</t>
+        </is>
+      </c>
+      <c r="C1072" t="inlineStr">
+        <is>
+          <t>Bajaj BJK 95I</t>
+        </is>
+      </c>
+      <c r="D1072" t="inlineStr">
+        <is>
+          <t>BJK95I</t>
+        </is>
+      </c>
+      <c r="H1072" t="n">
+        <v>420000</v>
+      </c>
+      <c r="I1072" t="n">
+        <v>420000</v>
+      </c>
+      <c r="J1072" t="inlineStr">
+        <is>
+          <t>efectivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="1073">
+      <c r="A1073" s="3" t="n">
+        <v>46117</v>
+      </c>
+      <c r="B1073" t="inlineStr">
+        <is>
+          <t>Donita Juan Camilo</t>
+        </is>
+      </c>
+      <c r="C1073" t="inlineStr">
+        <is>
+          <t>Bajaj BJK 95I</t>
+        </is>
+      </c>
+      <c r="D1073" t="inlineStr">
+        <is>
+          <t>BJK95I</t>
+        </is>
+      </c>
+      <c r="H1073" t="n">
+        <v>420000</v>
+      </c>
+      <c r="I1073" t="n">
+        <v>420000</v>
+      </c>
+      <c r="J1073" t="inlineStr">
+        <is>
+          <t>efectivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="1074">
+      <c r="A1074" s="3" t="n">
+        <v>46147</v>
+      </c>
+      <c r="B1074" t="inlineStr">
+        <is>
+          <t>Donita Juan Camilo</t>
+        </is>
+      </c>
+      <c r="C1074" t="inlineStr">
+        <is>
+          <t>Bajaj BJK 95I</t>
+        </is>
+      </c>
+      <c r="D1074" t="inlineStr">
+        <is>
+          <t>BJK95I</t>
+        </is>
+      </c>
+      <c r="H1074" t="n">
+        <v>420000</v>
+      </c>
+      <c r="I1074" t="n">
+        <v>420000</v>
+      </c>
+      <c r="J1074" t="inlineStr">
+        <is>
+          <t>efectivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="1075">
+      <c r="A1075" s="3" t="n">
+        <v>46175</v>
+      </c>
+      <c r="B1075" t="inlineStr">
+        <is>
+          <t>Donita Juan Camilo</t>
+        </is>
+      </c>
+      <c r="C1075" t="inlineStr">
+        <is>
+          <t>Bajaj BJK 95I</t>
+        </is>
+      </c>
+      <c r="D1075" t="inlineStr">
+        <is>
+          <t>BJK95I</t>
+        </is>
+      </c>
+      <c r="H1075" t="n">
+        <v>420000</v>
+      </c>
+      <c r="I1075" t="n">
+        <v>420000</v>
+      </c>
+      <c r="J1075" t="inlineStr">
+        <is>
+          <t>efectivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="1076">
+      <c r="A1076" s="3" t="n">
+        <v>46123</v>
+      </c>
+      <c r="B1076" t="inlineStr">
+        <is>
+          <t>Alejandra</t>
+        </is>
+      </c>
+      <c r="C1076" t="inlineStr">
+        <is>
+          <t>Bajaj OKS 30I</t>
+        </is>
+      </c>
+      <c r="D1076" t="inlineStr">
+        <is>
+          <t>OKS30I</t>
+        </is>
+      </c>
+      <c r="H1076" t="n">
+        <v>240000</v>
+      </c>
+      <c r="I1076" t="n">
+        <v>240000</v>
+      </c>
+      <c r="J1076" t="inlineStr">
+        <is>
+          <t>efectivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="1077">
+      <c r="A1077" s="3" t="n">
+        <v>46135</v>
+      </c>
+      <c r="B1077" t="inlineStr">
+        <is>
+          <t>Alejandra</t>
+        </is>
+      </c>
+      <c r="C1077" t="inlineStr">
+        <is>
+          <t>Bajaj OKS 30I</t>
+        </is>
+      </c>
+      <c r="D1077" t="inlineStr">
+        <is>
+          <t>OKS30I</t>
+        </is>
+      </c>
+      <c r="H1077" t="n">
+        <v>240000</v>
+      </c>
+      <c r="I1077" t="n">
+        <v>240000</v>
+      </c>
+      <c r="J1077" t="inlineStr">
+        <is>
+          <t>efectivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="1078">
+      <c r="A1078" s="3" t="n">
+        <v>46144</v>
+      </c>
+      <c r="B1078" t="inlineStr">
+        <is>
+          <t>Alejandra</t>
+        </is>
+      </c>
+      <c r="C1078" t="inlineStr">
+        <is>
+          <t>Bajaj OKS 30I</t>
+        </is>
+      </c>
+      <c r="D1078" t="inlineStr">
+        <is>
+          <t>OKS30I</t>
+        </is>
+      </c>
+      <c r="H1078" t="n">
+        <v>240000</v>
+      </c>
+      <c r="I1078" t="n">
+        <v>240000</v>
+      </c>
+      <c r="J1078" t="inlineStr">
+        <is>
+          <t>efectivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="1079">
+      <c r="A1079" s="3" t="n">
+        <v>46151</v>
+      </c>
+      <c r="B1079" t="inlineStr">
+        <is>
+          <t>Alejandra</t>
+        </is>
+      </c>
+      <c r="C1079" t="inlineStr">
+        <is>
+          <t>Bajaj OKS 30I</t>
+        </is>
+      </c>
+      <c r="D1079" t="inlineStr">
+        <is>
+          <t>OKS30I</t>
+        </is>
+      </c>
+      <c r="H1079" t="n">
+        <v>240000</v>
+      </c>
+      <c r="I1079" t="n">
+        <v>240000</v>
+      </c>
+      <c r="J1079" t="inlineStr">
+        <is>
+          <t>efectivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="1080">
+      <c r="A1080" s="3" t="n">
+        <v>46158</v>
+      </c>
+      <c r="B1080" t="inlineStr">
+        <is>
+          <t>Alejandra</t>
+        </is>
+      </c>
+      <c r="C1080" t="inlineStr">
+        <is>
+          <t>Bajaj OKS 30I</t>
+        </is>
+      </c>
+      <c r="D1080" t="inlineStr">
+        <is>
+          <t>OKS30I</t>
+        </is>
+      </c>
+      <c r="H1080" t="n">
+        <v>240000</v>
+      </c>
+      <c r="I1080" t="n">
+        <v>240000</v>
+      </c>
+      <c r="J1080" t="inlineStr">
+        <is>
+          <t>efectivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="1081">
+      <c r="A1081" s="3" t="n">
+        <v>46166</v>
+      </c>
+      <c r="B1081" t="inlineStr">
+        <is>
+          <t>Alejandra</t>
+        </is>
+      </c>
+      <c r="C1081" t="inlineStr">
+        <is>
+          <t>Bajaj OKS 30I</t>
+        </is>
+      </c>
+      <c r="D1081" t="inlineStr">
+        <is>
+          <t>OKS30I</t>
+        </is>
+      </c>
+      <c r="H1081" t="n">
+        <v>240000</v>
+      </c>
+      <c r="I1081" t="n">
+        <v>240000</v>
+      </c>
+      <c r="J1081" t="inlineStr">
+        <is>
+          <t>efectivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="1082">
+      <c r="A1082" s="3" t="n">
+        <v>46174</v>
+      </c>
+      <c r="B1082" t="inlineStr">
+        <is>
+          <t>Alejandra</t>
+        </is>
+      </c>
+      <c r="C1082" t="inlineStr">
+        <is>
+          <t>Bajaj OKS 30I</t>
+        </is>
+      </c>
+      <c r="D1082" t="inlineStr">
+        <is>
+          <t>OKS30I</t>
+        </is>
+      </c>
+      <c r="H1082" t="n">
+        <v>240000</v>
+      </c>
+      <c r="I1082" t="n">
+        <v>240000</v>
+      </c>
+      <c r="J1082" t="inlineStr">
+        <is>
+          <t>efectivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="1083">
+      <c r="A1083" s="3" t="n">
+        <v>46182</v>
+      </c>
+      <c r="B1083" t="inlineStr">
+        <is>
+          <t>Alejandra</t>
+        </is>
+      </c>
+      <c r="C1083" t="inlineStr">
+        <is>
+          <t>Bajaj OKS 30I</t>
+        </is>
+      </c>
+      <c r="D1083" t="inlineStr">
+        <is>
+          <t>OKS30I</t>
+        </is>
+      </c>
+      <c r="H1083" t="n">
+        <v>240000</v>
+      </c>
+      <c r="I1083" t="n">
+        <v>240000</v>
+      </c>
+      <c r="J1083" t="inlineStr">
+        <is>
+          <t>efectivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="1084">
+      <c r="A1084" s="3" t="n">
+        <v>46189</v>
+      </c>
+      <c r="B1084" t="inlineStr">
+        <is>
+          <t>Alejandra</t>
+        </is>
+      </c>
+      <c r="C1084" t="inlineStr">
+        <is>
+          <t>Bajaj OKS 30I</t>
+        </is>
+      </c>
+      <c r="D1084" t="inlineStr">
+        <is>
+          <t>OKS30I</t>
+        </is>
+      </c>
+      <c r="H1084" t="n">
+        <v>240000</v>
+      </c>
+      <c r="I1084" t="n">
+        <v>240000</v>
+      </c>
+      <c r="J1084" t="inlineStr">
+        <is>
+          <t>efectivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="1085">
+      <c r="A1085" s="3" t="n">
+        <v>46197</v>
+      </c>
+      <c r="B1085" t="inlineStr">
+        <is>
+          <t>Alejandra</t>
+        </is>
+      </c>
+      <c r="C1085" t="inlineStr">
+        <is>
+          <t>Bajaj OKS 30I</t>
+        </is>
+      </c>
+      <c r="D1085" t="inlineStr">
+        <is>
+          <t>OKS30I</t>
+        </is>
+      </c>
+      <c r="H1085" t="n">
+        <v>240000</v>
+      </c>
+      <c r="I1085" t="n">
+        <v>240000</v>
+      </c>
+      <c r="J1085" t="inlineStr">
+        <is>
+          <t>efectivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="1086">
+      <c r="A1086" s="3" t="n">
+        <v>46204</v>
+      </c>
+      <c r="B1086" t="inlineStr">
+        <is>
+          <t>Alejandra</t>
+        </is>
+      </c>
+      <c r="C1086" t="inlineStr">
+        <is>
+          <t>Bajaj OKS 30I</t>
+        </is>
+      </c>
+      <c r="D1086" t="inlineStr">
+        <is>
+          <t>OKS30I</t>
+        </is>
+      </c>
+      <c r="H1086" t="n">
+        <v>240000</v>
+      </c>
+      <c r="I1086" t="n">
+        <v>240000</v>
+      </c>
+      <c r="J1086" t="inlineStr">
+        <is>
+          <t>efectivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="1087">
+      <c r="A1087" s="3" t="n">
+        <v>46210</v>
+      </c>
+      <c r="B1087" t="inlineStr">
+        <is>
+          <t>Alejandra</t>
+        </is>
+      </c>
+      <c r="C1087" t="inlineStr">
+        <is>
+          <t>Bajaj OKS 30I</t>
+        </is>
+      </c>
+      <c r="D1087" t="inlineStr">
+        <is>
+          <t>OKS30I</t>
+        </is>
+      </c>
+      <c r="H1087" t="n">
+        <v>240000</v>
+      </c>
+      <c r="I1087" t="n">
+        <v>240000</v>
+      </c>
+      <c r="J1087" t="inlineStr">
+        <is>
+          <t>efectivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="1088">
+      <c r="A1088" s="3" t="n">
+        <v>46216</v>
+      </c>
+      <c r="B1088" t="inlineStr">
+        <is>
+          <t>Alejandra</t>
+        </is>
+      </c>
+      <c r="C1088" t="inlineStr">
+        <is>
+          <t>Bajaj OKS 30I</t>
+        </is>
+      </c>
+      <c r="D1088" t="inlineStr">
+        <is>
+          <t>OKS30I</t>
+        </is>
+      </c>
+      <c r="H1088" t="n">
+        <v>240000</v>
+      </c>
+      <c r="I1088" t="n">
+        <v>240000</v>
+      </c>
+      <c r="J1088" t="inlineStr">
         <is>
           <t>efectivo</t>
         </is>

</xml_diff>

<commit_message>
feat: agregar fotos 46-49 (Carlos, Francisco, Yesenia, Alvania)
Carlos (BLB45I): 18 meses / 72 cuotas, 4 pagos may-jun 2026
Francisco Buñuelo (BLG78I): 24 meses / 48 cuotas bisemanales, tarifa 190k, 4 pagos
Yesenia (HWO62I): 18 meses / 72 cuotas, 3 pagos jul 2026
Alvania (HWD78I): 18 meses / 72 cuotas, 2 pagos jul 2026

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/control_motos_tio.xlsx
+++ b/control_motos_tio.xlsx
@@ -565,7 +565,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F28"/>
+  <dimension ref="A1:F32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -1364,6 +1364,118 @@
         <v>84</v>
       </c>
     </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Carlos</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Bajaj BLB 45I</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>BLB45I</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="n">
+        <v>46158</v>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Foto 46 | 18 meses | 72 cuotas | 4 pagos registrados | moto #29</t>
+        </is>
+      </c>
+      <c r="F29" t="n">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Francisco (Buñuelo)</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Bajaj BLG 78I</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>BLG78I</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="n">
+        <v>46145</v>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Foto 47 | 24 meses | 48 cuotas bisemanales | tarifa 190.000 | 4 pagos | moto #30</t>
+        </is>
+      </c>
+      <c r="F30" t="n">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Yesenia</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Bajaj HWO 62I</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>HWO62I</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="n">
+        <v>46211</v>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Foto 48 | 18 meses | 72 cuotas | 3 pagos registrados | moto #31</t>
+        </is>
+      </c>
+      <c r="F31" t="n">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Alvania</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Bajaj HWD 78I</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>HWD78I</t>
+        </is>
+      </c>
+      <c r="D32" s="2" t="n">
+        <v>46213</v>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>Foto 49 | 18 meses | 72 cuotas | 2 pagos registrados | moto #32</t>
+        </is>
+      </c>
+      <c r="F32" t="n">
+        <v>72</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1375,7 +1487,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P1088"/>
+  <dimension ref="A1:P1101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -35135,6 +35247,409 @@
         <v>240000</v>
       </c>
       <c r="J1088" t="inlineStr">
+        <is>
+          <t>efectivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="1089">
+      <c r="A1089" s="3" t="n">
+        <v>46158</v>
+      </c>
+      <c r="B1089" t="inlineStr">
+        <is>
+          <t>Carlos</t>
+        </is>
+      </c>
+      <c r="C1089" t="inlineStr">
+        <is>
+          <t>Bajaj BLB 45I</t>
+        </is>
+      </c>
+      <c r="D1089" t="inlineStr">
+        <is>
+          <t>BLB45I</t>
+        </is>
+      </c>
+      <c r="H1089" t="n">
+        <v>240000</v>
+      </c>
+      <c r="I1089" t="n">
+        <v>240000</v>
+      </c>
+      <c r="J1089" t="inlineStr">
+        <is>
+          <t>efectivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="1090">
+      <c r="A1090" s="3" t="n">
+        <v>46166</v>
+      </c>
+      <c r="B1090" t="inlineStr">
+        <is>
+          <t>Carlos</t>
+        </is>
+      </c>
+      <c r="C1090" t="inlineStr">
+        <is>
+          <t>Bajaj BLB 45I</t>
+        </is>
+      </c>
+      <c r="D1090" t="inlineStr">
+        <is>
+          <t>BLB45I</t>
+        </is>
+      </c>
+      <c r="H1090" t="n">
+        <v>240000</v>
+      </c>
+      <c r="I1090" t="n">
+        <v>240000</v>
+      </c>
+      <c r="J1090" t="inlineStr">
+        <is>
+          <t>efectivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="1091">
+      <c r="A1091" s="3" t="n">
+        <v>46177</v>
+      </c>
+      <c r="B1091" t="inlineStr">
+        <is>
+          <t>Carlos</t>
+        </is>
+      </c>
+      <c r="C1091" t="inlineStr">
+        <is>
+          <t>Bajaj BLB 45I</t>
+        </is>
+      </c>
+      <c r="D1091" t="inlineStr">
+        <is>
+          <t>BLB45I</t>
+        </is>
+      </c>
+      <c r="H1091" t="n">
+        <v>240000</v>
+      </c>
+      <c r="I1091" t="n">
+        <v>240000</v>
+      </c>
+      <c r="J1091" t="inlineStr">
+        <is>
+          <t>efectivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="1092">
+      <c r="A1092" s="3" t="n">
+        <v>46191</v>
+      </c>
+      <c r="B1092" t="inlineStr">
+        <is>
+          <t>Carlos</t>
+        </is>
+      </c>
+      <c r="C1092" t="inlineStr">
+        <is>
+          <t>Bajaj BLB 45I</t>
+        </is>
+      </c>
+      <c r="D1092" t="inlineStr">
+        <is>
+          <t>BLB45I</t>
+        </is>
+      </c>
+      <c r="H1092" t="n">
+        <v>240000</v>
+      </c>
+      <c r="I1092" t="n">
+        <v>240000</v>
+      </c>
+      <c r="J1092" t="inlineStr">
+        <is>
+          <t>efectivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="1093">
+      <c r="A1093" s="3" t="n">
+        <v>46145</v>
+      </c>
+      <c r="B1093" t="inlineStr">
+        <is>
+          <t>Francisco (Buñuelo)</t>
+        </is>
+      </c>
+      <c r="C1093" t="inlineStr">
+        <is>
+          <t>Bajaj BLG 78I</t>
+        </is>
+      </c>
+      <c r="D1093" t="inlineStr">
+        <is>
+          <t>BLG78I</t>
+        </is>
+      </c>
+      <c r="H1093" t="n">
+        <v>190000</v>
+      </c>
+      <c r="I1093" t="n">
+        <v>190000</v>
+      </c>
+      <c r="J1093" t="inlineStr">
+        <is>
+          <t>efectivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="1094">
+      <c r="A1094" s="3" t="n">
+        <v>46157</v>
+      </c>
+      <c r="B1094" t="inlineStr">
+        <is>
+          <t>Francisco (Buñuelo)</t>
+        </is>
+      </c>
+      <c r="C1094" t="inlineStr">
+        <is>
+          <t>Bajaj BLG 78I</t>
+        </is>
+      </c>
+      <c r="D1094" t="inlineStr">
+        <is>
+          <t>BLG78I</t>
+        </is>
+      </c>
+      <c r="H1094" t="n">
+        <v>190000</v>
+      </c>
+      <c r="I1094" t="n">
+        <v>190000</v>
+      </c>
+      <c r="J1094" t="inlineStr">
+        <is>
+          <t>efectivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="1095">
+      <c r="A1095" s="3" t="n">
+        <v>46172</v>
+      </c>
+      <c r="B1095" t="inlineStr">
+        <is>
+          <t>Francisco (Buñuelo)</t>
+        </is>
+      </c>
+      <c r="C1095" t="inlineStr">
+        <is>
+          <t>Bajaj BLG 78I</t>
+        </is>
+      </c>
+      <c r="D1095" t="inlineStr">
+        <is>
+          <t>BLG78I</t>
+        </is>
+      </c>
+      <c r="H1095" t="n">
+        <v>190000</v>
+      </c>
+      <c r="I1095" t="n">
+        <v>190000</v>
+      </c>
+      <c r="J1095" t="inlineStr">
+        <is>
+          <t>efectivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="1096">
+      <c r="A1096" s="3" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B1096" t="inlineStr">
+        <is>
+          <t>Francisco (Buñuelo)</t>
+        </is>
+      </c>
+      <c r="C1096" t="inlineStr">
+        <is>
+          <t>Bajaj BLG 78I</t>
+        </is>
+      </c>
+      <c r="D1096" t="inlineStr">
+        <is>
+          <t>BLG78I</t>
+        </is>
+      </c>
+      <c r="H1096" t="n">
+        <v>190000</v>
+      </c>
+      <c r="I1096" t="n">
+        <v>190000</v>
+      </c>
+      <c r="J1096" t="inlineStr">
+        <is>
+          <t>efectivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="1097">
+      <c r="A1097" s="3" t="n">
+        <v>46211</v>
+      </c>
+      <c r="B1097" t="inlineStr">
+        <is>
+          <t>Yesenia</t>
+        </is>
+      </c>
+      <c r="C1097" t="inlineStr">
+        <is>
+          <t>Bajaj HWO 62I</t>
+        </is>
+      </c>
+      <c r="D1097" t="inlineStr">
+        <is>
+          <t>HWO62I</t>
+        </is>
+      </c>
+      <c r="H1097" t="n">
+        <v>240000</v>
+      </c>
+      <c r="I1097" t="n">
+        <v>240000</v>
+      </c>
+      <c r="J1097" t="inlineStr">
+        <is>
+          <t>efectivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="1098">
+      <c r="A1098" s="3" t="n">
+        <v>46218</v>
+      </c>
+      <c r="B1098" t="inlineStr">
+        <is>
+          <t>Yesenia</t>
+        </is>
+      </c>
+      <c r="C1098" t="inlineStr">
+        <is>
+          <t>Bajaj HWO 62I</t>
+        </is>
+      </c>
+      <c r="D1098" t="inlineStr">
+        <is>
+          <t>HWO62I</t>
+        </is>
+      </c>
+      <c r="H1098" t="n">
+        <v>240000</v>
+      </c>
+      <c r="I1098" t="n">
+        <v>240000</v>
+      </c>
+      <c r="J1098" t="inlineStr">
+        <is>
+          <t>efectivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="1099">
+      <c r="A1099" s="3" t="n">
+        <v>46225</v>
+      </c>
+      <c r="B1099" t="inlineStr">
+        <is>
+          <t>Yesenia</t>
+        </is>
+      </c>
+      <c r="C1099" t="inlineStr">
+        <is>
+          <t>Bajaj HWO 62I</t>
+        </is>
+      </c>
+      <c r="D1099" t="inlineStr">
+        <is>
+          <t>HWO62I</t>
+        </is>
+      </c>
+      <c r="H1099" t="n">
+        <v>240000</v>
+      </c>
+      <c r="I1099" t="n">
+        <v>240000</v>
+      </c>
+      <c r="J1099" t="inlineStr">
+        <is>
+          <t>efectivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="1100">
+      <c r="A1100" s="3" t="n">
+        <v>46213</v>
+      </c>
+      <c r="B1100" t="inlineStr">
+        <is>
+          <t>Alvania</t>
+        </is>
+      </c>
+      <c r="C1100" t="inlineStr">
+        <is>
+          <t>Bajaj HWD 78I</t>
+        </is>
+      </c>
+      <c r="D1100" t="inlineStr">
+        <is>
+          <t>HWD78I</t>
+        </is>
+      </c>
+      <c r="H1100" t="n">
+        <v>240000</v>
+      </c>
+      <c r="I1100" t="n">
+        <v>240000</v>
+      </c>
+      <c r="J1100" t="inlineStr">
+        <is>
+          <t>efectivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="1101">
+      <c r="A1101" s="3" t="n">
+        <v>46220</v>
+      </c>
+      <c r="B1101" t="inlineStr">
+        <is>
+          <t>Alvania</t>
+        </is>
+      </c>
+      <c r="C1101" t="inlineStr">
+        <is>
+          <t>Bajaj HWD 78I</t>
+        </is>
+      </c>
+      <c r="D1101" t="inlineStr">
+        <is>
+          <t>HWD78I</t>
+        </is>
+      </c>
+      <c r="H1101" t="n">
+        <v>240000</v>
+      </c>
+      <c r="I1101" t="n">
+        <v>240000</v>
+      </c>
+      <c r="J1101" t="inlineStr">
         <is>
           <t>efectivo</t>
         </is>

</xml_diff>

<commit_message>
feat: agregar foto 50 — Yurais Polo HWM 11I (cliente nuevo sin pagos)
Moto #33, 18 meses / 72 cuotas — pagina en blanco, primer pago pendiente

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/control_motos_tio.xlsx
+++ b/control_motos_tio.xlsx
@@ -565,7 +565,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F32"/>
+  <dimension ref="A1:F33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -1473,6 +1473,34 @@
         </is>
       </c>
       <c r="F32" t="n">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Yurais Polo</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Bajaj HWM 11I</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>HWM11I</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="n">
+        <v>46235</v>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Foto 50 | 18 meses | 72 cuotas | moto #33 | SIN PAGOS aun — cliente nuevo</t>
+        </is>
+      </c>
+      <c r="F33" t="n">
         <v>72</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Corrige placa de Dorlys: EYO114 → EYO11H
</commit_message>
<xml_diff>
--- a/control_motos_tio.xlsx
+++ b/control_motos_tio.xlsx
@@ -616,12 +616,12 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Bajaj EYO 114</t>
+          <t>Bajaj EYO 11H</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>EYO114</t>
+          <t>EYO11H</t>
         </is>
       </c>
       <c r="D2" s="2" t="n">
@@ -1622,12 +1622,12 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Bajaj EYO 114</t>
+          <t>Bajaj EYO 11H</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>EYO114</t>
+          <t>EYO11H</t>
         </is>
       </c>
       <c r="H2" t="n">
@@ -1653,12 +1653,12 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Bajaj EYO 114</t>
+          <t>Bajaj EYO 11H</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>EYO114</t>
+          <t>EYO11H</t>
         </is>
       </c>
       <c r="H3" t="n">
@@ -1684,12 +1684,12 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Bajaj EYO 114</t>
+          <t>Bajaj EYO 11H</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>EYO114</t>
+          <t>EYO11H</t>
         </is>
       </c>
       <c r="H4" t="n">
@@ -1715,12 +1715,12 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Bajaj EYO 114</t>
+          <t>Bajaj EYO 11H</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>EYO114</t>
+          <t>EYO11H</t>
         </is>
       </c>
       <c r="H5" t="n">
@@ -1746,12 +1746,12 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Bajaj EYO 114</t>
+          <t>Bajaj EYO 11H</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>EYO114</t>
+          <t>EYO11H</t>
         </is>
       </c>
       <c r="H6" t="n">
@@ -1777,12 +1777,12 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Bajaj EYO 114</t>
+          <t>Bajaj EYO 11H</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>EYO114</t>
+          <t>EYO11H</t>
         </is>
       </c>
       <c r="H7" t="n">
@@ -1808,12 +1808,12 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Bajaj EYO 114</t>
+          <t>Bajaj EYO 11H</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>EYO114</t>
+          <t>EYO11H</t>
         </is>
       </c>
       <c r="H8" t="n">
@@ -1839,12 +1839,12 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Bajaj EYO 114</t>
+          <t>Bajaj EYO 11H</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>EYO114</t>
+          <t>EYO11H</t>
         </is>
       </c>
       <c r="H9" t="n">
@@ -1870,12 +1870,12 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Bajaj EYO 114</t>
+          <t>Bajaj EYO 11H</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>EYO114</t>
+          <t>EYO11H</t>
         </is>
       </c>
       <c r="H10" t="n">
@@ -1901,12 +1901,12 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Bajaj EYO 114</t>
+          <t>Bajaj EYO 11H</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>EYO114</t>
+          <t>EYO11H</t>
         </is>
       </c>
       <c r="H11" t="n">
@@ -1932,12 +1932,12 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Bajaj EYO 114</t>
+          <t>Bajaj EYO 11H</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>EYO114</t>
+          <t>EYO11H</t>
         </is>
       </c>
       <c r="H12" t="n">
@@ -1963,12 +1963,12 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Bajaj EYO 114</t>
+          <t>Bajaj EYO 11H</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>EYO114</t>
+          <t>EYO11H</t>
         </is>
       </c>
       <c r="H13" t="n">
@@ -1994,12 +1994,12 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Bajaj EYO 114</t>
+          <t>Bajaj EYO 11H</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>EYO114</t>
+          <t>EYO11H</t>
         </is>
       </c>
       <c r="H14" t="n">
@@ -2025,12 +2025,12 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Bajaj EYO 114</t>
+          <t>Bajaj EYO 11H</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>EYO114</t>
+          <t>EYO11H</t>
         </is>
       </c>
       <c r="H15" t="n">
@@ -2056,12 +2056,12 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Bajaj EYO 114</t>
+          <t>Bajaj EYO 11H</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>EYO114</t>
+          <t>EYO11H</t>
         </is>
       </c>
       <c r="H16" t="n">
@@ -2087,12 +2087,12 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Bajaj EYO 114</t>
+          <t>Bajaj EYO 11H</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>EYO114</t>
+          <t>EYO11H</t>
         </is>
       </c>
       <c r="H17" t="n">
@@ -2118,12 +2118,12 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Bajaj EYO 114</t>
+          <t>Bajaj EYO 11H</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>EYO114</t>
+          <t>EYO11H</t>
         </is>
       </c>
       <c r="H18" t="n">
@@ -2149,12 +2149,12 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Bajaj EYO 114</t>
+          <t>Bajaj EYO 11H</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>EYO114</t>
+          <t>EYO11H</t>
         </is>
       </c>
       <c r="H19" t="n">
@@ -2180,12 +2180,12 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Bajaj EYO 114</t>
+          <t>Bajaj EYO 11H</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>EYO114</t>
+          <t>EYO11H</t>
         </is>
       </c>
       <c r="H20" t="n">
@@ -2211,12 +2211,12 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Bajaj EYO 114</t>
+          <t>Bajaj EYO 11H</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>EYO114</t>
+          <t>EYO11H</t>
         </is>
       </c>
       <c r="H21" t="n">
@@ -2242,12 +2242,12 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Bajaj EYO 114</t>
+          <t>Bajaj EYO 11H</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>EYO114</t>
+          <t>EYO11H</t>
         </is>
       </c>
       <c r="H22" t="n">
@@ -2273,12 +2273,12 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Bajaj EYO 114</t>
+          <t>Bajaj EYO 11H</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>EYO114</t>
+          <t>EYO11H</t>
         </is>
       </c>
       <c r="H23" t="n">
@@ -2304,12 +2304,12 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Bajaj EYO 114</t>
+          <t>Bajaj EYO 11H</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>EYO114</t>
+          <t>EYO11H</t>
         </is>
       </c>
       <c r="H24" t="n">
@@ -2335,12 +2335,12 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Bajaj EYO 114</t>
+          <t>Bajaj EYO 11H</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>EYO114</t>
+          <t>EYO11H</t>
         </is>
       </c>
       <c r="H25" t="n">
@@ -2366,12 +2366,12 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Bajaj EYO 114</t>
+          <t>Bajaj EYO 11H</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>EYO114</t>
+          <t>EYO11H</t>
         </is>
       </c>
       <c r="H26" t="n">
@@ -2397,12 +2397,12 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Bajaj EYO 114</t>
+          <t>Bajaj EYO 11H</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>EYO114</t>
+          <t>EYO11H</t>
         </is>
       </c>
       <c r="H27" t="n">
@@ -2428,12 +2428,12 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Bajaj EYO 114</t>
+          <t>Bajaj EYO 11H</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>EYO114</t>
+          <t>EYO11H</t>
         </is>
       </c>
       <c r="H28" t="n">
@@ -2459,12 +2459,12 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Bajaj EYO 114</t>
+          <t>Bajaj EYO 11H</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>EYO114</t>
+          <t>EYO11H</t>
         </is>
       </c>
       <c r="H29" t="n">
@@ -2490,12 +2490,12 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Bajaj EYO 114</t>
+          <t>Bajaj EYO 11H</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>EYO114</t>
+          <t>EYO11H</t>
         </is>
       </c>
       <c r="H30" t="n">
@@ -2521,12 +2521,12 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Bajaj EYO 114</t>
+          <t>Bajaj EYO 11H</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>EYO114</t>
+          <t>EYO11H</t>
         </is>
       </c>
       <c r="H31" t="n">
@@ -2552,12 +2552,12 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Bajaj EYO 114</t>
+          <t>Bajaj EYO 11H</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>EYO114</t>
+          <t>EYO11H</t>
         </is>
       </c>
       <c r="H32" t="n">
@@ -2583,12 +2583,12 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Bajaj EYO 114</t>
+          <t>Bajaj EYO 11H</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>EYO114</t>
+          <t>EYO11H</t>
         </is>
       </c>
       <c r="H33" t="n">
@@ -2614,12 +2614,12 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Bajaj EYO 114</t>
+          <t>Bajaj EYO 11H</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>EYO114</t>
+          <t>EYO11H</t>
         </is>
       </c>
       <c r="H34" t="n">
@@ -2645,12 +2645,12 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Bajaj EYO 114</t>
+          <t>Bajaj EYO 11H</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>EYO114</t>
+          <t>EYO11H</t>
         </is>
       </c>
       <c r="H35" t="n">
@@ -2676,12 +2676,12 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Bajaj EYO 114</t>
+          <t>Bajaj EYO 11H</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>EYO114</t>
+          <t>EYO11H</t>
         </is>
       </c>
       <c r="H36" t="n">
@@ -2707,12 +2707,12 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Bajaj EYO 114</t>
+          <t>Bajaj EYO 11H</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>EYO114</t>
+          <t>EYO11H</t>
         </is>
       </c>
       <c r="H37" t="n">
@@ -2738,12 +2738,12 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Bajaj EYO 114</t>
+          <t>Bajaj EYO 11H</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>EYO114</t>
+          <t>EYO11H</t>
         </is>
       </c>
       <c r="H38" t="n">
@@ -2769,12 +2769,12 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Bajaj EYO 114</t>
+          <t>Bajaj EYO 11H</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>EYO114</t>
+          <t>EYO11H</t>
         </is>
       </c>
       <c r="H39" t="n">
@@ -2800,12 +2800,12 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Bajaj EYO 114</t>
+          <t>Bajaj EYO 11H</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>EYO114</t>
+          <t>EYO11H</t>
         </is>
       </c>
       <c r="H40" t="n">
@@ -2831,12 +2831,12 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Bajaj EYO 114</t>
+          <t>Bajaj EYO 11H</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>EYO114</t>
+          <t>EYO11H</t>
         </is>
       </c>
       <c r="H41" t="n">
@@ -2862,12 +2862,12 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Bajaj EYO 114</t>
+          <t>Bajaj EYO 11H</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>EYO114</t>
+          <t>EYO11H</t>
         </is>
       </c>
       <c r="H42" t="n">
@@ -2893,12 +2893,12 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Bajaj EYO 114</t>
+          <t>Bajaj EYO 11H</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>EYO114</t>
+          <t>EYO11H</t>
         </is>
       </c>
       <c r="H43" t="n">
@@ -2924,12 +2924,12 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Bajaj EYO 114</t>
+          <t>Bajaj EYO 11H</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>EYO114</t>
+          <t>EYO11H</t>
         </is>
       </c>
       <c r="H44" t="n">
@@ -2955,12 +2955,12 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Bajaj EYO 114</t>
+          <t>Bajaj EYO 11H</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>EYO114</t>
+          <t>EYO11H</t>
         </is>
       </c>
       <c r="H45" t="n">
@@ -2986,12 +2986,12 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Bajaj EYO 114</t>
+          <t>Bajaj EYO 11H</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>EYO114</t>
+          <t>EYO11H</t>
         </is>
       </c>
       <c r="H46" t="n">
@@ -3017,12 +3017,12 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Bajaj EYO 114</t>
+          <t>Bajaj EYO 11H</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>EYO114</t>
+          <t>EYO11H</t>
         </is>
       </c>
       <c r="H47" t="n">
@@ -3048,12 +3048,12 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Bajaj EYO 114</t>
+          <t>Bajaj EYO 11H</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>EYO114</t>
+          <t>EYO11H</t>
         </is>
       </c>
       <c r="H48" t="n">
@@ -3079,12 +3079,12 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Bajaj EYO 114</t>
+          <t>Bajaj EYO 11H</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>EYO114</t>
+          <t>EYO11H</t>
         </is>
       </c>
       <c r="H49" t="n">
@@ -3110,12 +3110,12 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Bajaj EYO 114</t>
+          <t>Bajaj EYO 11H</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>EYO114</t>
+          <t>EYO11H</t>
         </is>
       </c>
       <c r="H50" t="n">
@@ -3141,12 +3141,12 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Bajaj EYO 114</t>
+          <t>Bajaj EYO 11H</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>EYO114</t>
+          <t>EYO11H</t>
         </is>
       </c>
       <c r="H51" t="n">
@@ -3172,12 +3172,12 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Bajaj EYO 114</t>
+          <t>Bajaj EYO 11H</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>EYO114</t>
+          <t>EYO11H</t>
         </is>
       </c>
       <c r="H52" t="n">
@@ -3203,12 +3203,12 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Bajaj EYO 114</t>
+          <t>Bajaj EYO 11H</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>EYO114</t>
+          <t>EYO11H</t>
         </is>
       </c>
       <c r="H53" t="n">
@@ -3234,12 +3234,12 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Bajaj EYO 114</t>
+          <t>Bajaj EYO 11H</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>EYO114</t>
+          <t>EYO11H</t>
         </is>
       </c>
       <c r="H54" t="n">
@@ -3265,12 +3265,12 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Bajaj EYO 114</t>
+          <t>Bajaj EYO 11H</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>EYO114</t>
+          <t>EYO11H</t>
         </is>
       </c>
       <c r="H55" t="n">
@@ -3296,12 +3296,12 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Bajaj EYO 114</t>
+          <t>Bajaj EYO 11H</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>EYO114</t>
+          <t>EYO11H</t>
         </is>
       </c>
       <c r="H56" t="n">
@@ -3327,12 +3327,12 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Bajaj EYO 114</t>
+          <t>Bajaj EYO 11H</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>EYO114</t>
+          <t>EYO11H</t>
         </is>
       </c>
       <c r="H57" t="n">
@@ -3358,12 +3358,12 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Bajaj EYO 114</t>
+          <t>Bajaj EYO 11H</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>EYO114</t>
+          <t>EYO11H</t>
         </is>
       </c>
       <c r="H58" t="n">

</xml_diff>

<commit_message>
feat: rediseño premium + filtros de periodo + renombres de clientes
- Filtro DESDE/HASTA con botones rápidos (Ayer, Esta semana, Este mes, Histórico)
- Diseño premium: barras doradas en tickers, panel oscuro, botones pill
- Columna # (número) y Placa separada en tabla de cuentas de cobro
- Esperado del mes: proyección semanal real por cliente (no suma histórica)
- 12 renombres de clientes: Engelo Junior, Negro Maria Jose, Sr Pedro,
  Brayan, Erik, Katherine, Ana Milena-Juan David, Manuel Olga,
  Daniela Nuñez, Alejandro, Karluis, Yuranis Polo
- Agrega index.html (formulario cobrador) y carpeta Fotos/

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/control_motos_tio.xlsx
+++ b/control_motos_tio.xlsx
@@ -723,17 +723,17 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Luis Gabriel Polo</t>
+          <t>Engelo Junior</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Bajaj KOM 89H</t>
+          <t>Bajaj UYL 39H</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>KOM89H</t>
+          <t>UYL39H</t>
         </is>
       </c>
       <c r="D6" s="2" t="n">
@@ -975,7 +975,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Nabro Maria Jesse</t>
+          <t>Negro Maria Jose</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -1003,7 +1003,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Luis Katherin Estor</t>
+          <t>Sr Pedro</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
@@ -1087,7 +1087,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Braillon</t>
+          <t>Brayan</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1143,7 +1143,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Erzik</t>
+          <t>Erik</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -1199,7 +1199,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Gonzado Estherline</t>
+          <t>Katherine</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -1217,7 +1217,7 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Cuñado de Katherine | del Choco | Tel: 3205570847 | 21 meses | 20160000 total | 84 cuotas | subtotal cuaderno 11.520.000 (48 cuotas) | 41 registradas fotos 38+39</t>
+          <t>del Choco | Tel: 3205570847 | 21 meses | 20160000 total | 84 cuotas | subtotal cuaderno 11.520.000 (48 cuotas) | 41 registradas fotos 38+39</t>
         </is>
       </c>
       <c r="F23" t="n">
@@ -1227,7 +1227,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Ana Milena Juan Davit</t>
+          <t>Ana Milena-Juan David</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -1283,7 +1283,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Manuel Alga</t>
+          <t>Manuel Olga</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -1339,7 +1339,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Donita Juan Camilo</t>
+          <t>Daniela Nuñez</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -1367,7 +1367,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Alejandra</t>
+          <t>Alejandro</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -1395,7 +1395,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Carlos</t>
+          <t>Karluis</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1507,7 +1507,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Yurais Polo</t>
+          <t>Yuranis Polo</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -9119,17 +9119,17 @@
       </c>
       <c r="B244" t="inlineStr">
         <is>
-          <t>Luis Gabriel Polo</t>
+          <t>Engelo Junior</t>
         </is>
       </c>
       <c r="C244" t="inlineStr">
         <is>
-          <t>Bajaj KOM 89H</t>
+          <t>Bajaj UYL 39H</t>
         </is>
       </c>
       <c r="D244" t="inlineStr">
         <is>
-          <t>KOM89H</t>
+          <t>UYL39H</t>
         </is>
       </c>
       <c r="H244" t="n">
@@ -9150,17 +9150,17 @@
       </c>
       <c r="B245" t="inlineStr">
         <is>
-          <t>Luis Gabriel Polo</t>
+          <t>Engelo Junior</t>
         </is>
       </c>
       <c r="C245" t="inlineStr">
         <is>
-          <t>Bajaj KOM 89H</t>
+          <t>Bajaj UYL 39H</t>
         </is>
       </c>
       <c r="D245" t="inlineStr">
         <is>
-          <t>KOM89H</t>
+          <t>UYL39H</t>
         </is>
       </c>
       <c r="H245" t="n">
@@ -9181,17 +9181,17 @@
       </c>
       <c r="B246" t="inlineStr">
         <is>
-          <t>Luis Gabriel Polo</t>
+          <t>Engelo Junior</t>
         </is>
       </c>
       <c r="C246" t="inlineStr">
         <is>
-          <t>Bajaj KOM 89H</t>
+          <t>Bajaj UYL 39H</t>
         </is>
       </c>
       <c r="D246" t="inlineStr">
         <is>
-          <t>KOM89H</t>
+          <t>UYL39H</t>
         </is>
       </c>
       <c r="H246" t="n">
@@ -9212,17 +9212,17 @@
       </c>
       <c r="B247" t="inlineStr">
         <is>
-          <t>Luis Gabriel Polo</t>
+          <t>Engelo Junior</t>
         </is>
       </c>
       <c r="C247" t="inlineStr">
         <is>
-          <t>Bajaj KOM 89H</t>
+          <t>Bajaj UYL 39H</t>
         </is>
       </c>
       <c r="D247" t="inlineStr">
         <is>
-          <t>KOM89H</t>
+          <t>UYL39H</t>
         </is>
       </c>
       <c r="H247" t="n">
@@ -9243,17 +9243,17 @@
       </c>
       <c r="B248" t="inlineStr">
         <is>
-          <t>Luis Gabriel Polo</t>
+          <t>Engelo Junior</t>
         </is>
       </c>
       <c r="C248" t="inlineStr">
         <is>
-          <t>Bajaj KOM 89H</t>
+          <t>Bajaj UYL 39H</t>
         </is>
       </c>
       <c r="D248" t="inlineStr">
         <is>
-          <t>KOM89H</t>
+          <t>UYL39H</t>
         </is>
       </c>
       <c r="H248" t="n">
@@ -9274,17 +9274,17 @@
       </c>
       <c r="B249" t="inlineStr">
         <is>
-          <t>Luis Gabriel Polo</t>
+          <t>Engelo Junior</t>
         </is>
       </c>
       <c r="C249" t="inlineStr">
         <is>
-          <t>Bajaj KOM 89H</t>
+          <t>Bajaj UYL 39H</t>
         </is>
       </c>
       <c r="D249" t="inlineStr">
         <is>
-          <t>KOM89H</t>
+          <t>UYL39H</t>
         </is>
       </c>
       <c r="H249" t="n">
@@ -9305,17 +9305,17 @@
       </c>
       <c r="B250" t="inlineStr">
         <is>
-          <t>Luis Gabriel Polo</t>
+          <t>Engelo Junior</t>
         </is>
       </c>
       <c r="C250" t="inlineStr">
         <is>
-          <t>Bajaj KOM 89H</t>
+          <t>Bajaj UYL 39H</t>
         </is>
       </c>
       <c r="D250" t="inlineStr">
         <is>
-          <t>KOM89H</t>
+          <t>UYL39H</t>
         </is>
       </c>
       <c r="H250" t="n">
@@ -9336,17 +9336,17 @@
       </c>
       <c r="B251" t="inlineStr">
         <is>
-          <t>Luis Gabriel Polo</t>
+          <t>Engelo Junior</t>
         </is>
       </c>
       <c r="C251" t="inlineStr">
         <is>
-          <t>Bajaj KOM 89H</t>
+          <t>Bajaj UYL 39H</t>
         </is>
       </c>
       <c r="D251" t="inlineStr">
         <is>
-          <t>KOM89H</t>
+          <t>UYL39H</t>
         </is>
       </c>
       <c r="H251" t="n">
@@ -9367,17 +9367,17 @@
       </c>
       <c r="B252" t="inlineStr">
         <is>
-          <t>Luis Gabriel Polo</t>
+          <t>Engelo Junior</t>
         </is>
       </c>
       <c r="C252" t="inlineStr">
         <is>
-          <t>Bajaj KOM 89H</t>
+          <t>Bajaj UYL 39H</t>
         </is>
       </c>
       <c r="D252" t="inlineStr">
         <is>
-          <t>KOM89H</t>
+          <t>UYL39H</t>
         </is>
       </c>
       <c r="H252" t="n">
@@ -9398,17 +9398,17 @@
       </c>
       <c r="B253" t="inlineStr">
         <is>
-          <t>Luis Gabriel Polo</t>
+          <t>Engelo Junior</t>
         </is>
       </c>
       <c r="C253" t="inlineStr">
         <is>
-          <t>Bajaj KOM 89H</t>
+          <t>Bajaj UYL 39H</t>
         </is>
       </c>
       <c r="D253" t="inlineStr">
         <is>
-          <t>KOM89H</t>
+          <t>UYL39H</t>
         </is>
       </c>
       <c r="H253" t="n">
@@ -9429,17 +9429,17 @@
       </c>
       <c r="B254" t="inlineStr">
         <is>
-          <t>Luis Gabriel Polo</t>
+          <t>Engelo Junior</t>
         </is>
       </c>
       <c r="C254" t="inlineStr">
         <is>
-          <t>Bajaj KOM 89H</t>
+          <t>Bajaj UYL 39H</t>
         </is>
       </c>
       <c r="D254" t="inlineStr">
         <is>
-          <t>KOM89H</t>
+          <t>UYL39H</t>
         </is>
       </c>
       <c r="H254" t="n">
@@ -9460,17 +9460,17 @@
       </c>
       <c r="B255" t="inlineStr">
         <is>
-          <t>Luis Gabriel Polo</t>
+          <t>Engelo Junior</t>
         </is>
       </c>
       <c r="C255" t="inlineStr">
         <is>
-          <t>Bajaj KOM 89H</t>
+          <t>Bajaj UYL 39H</t>
         </is>
       </c>
       <c r="D255" t="inlineStr">
         <is>
-          <t>KOM89H</t>
+          <t>UYL39H</t>
         </is>
       </c>
       <c r="H255" t="n">
@@ -9491,17 +9491,17 @@
       </c>
       <c r="B256" t="inlineStr">
         <is>
-          <t>Luis Gabriel Polo</t>
+          <t>Engelo Junior</t>
         </is>
       </c>
       <c r="C256" t="inlineStr">
         <is>
-          <t>Bajaj KOM 89H</t>
+          <t>Bajaj UYL 39H</t>
         </is>
       </c>
       <c r="D256" t="inlineStr">
         <is>
-          <t>KOM89H</t>
+          <t>UYL39H</t>
         </is>
       </c>
       <c r="H256" t="n">
@@ -9522,17 +9522,17 @@
       </c>
       <c r="B257" t="inlineStr">
         <is>
-          <t>Luis Gabriel Polo</t>
+          <t>Engelo Junior</t>
         </is>
       </c>
       <c r="C257" t="inlineStr">
         <is>
-          <t>Bajaj KOM 89H</t>
+          <t>Bajaj UYL 39H</t>
         </is>
       </c>
       <c r="D257" t="inlineStr">
         <is>
-          <t>KOM89H</t>
+          <t>UYL39H</t>
         </is>
       </c>
       <c r="H257" t="n">
@@ -9553,17 +9553,17 @@
       </c>
       <c r="B258" t="inlineStr">
         <is>
-          <t>Luis Gabriel Polo</t>
+          <t>Engelo Junior</t>
         </is>
       </c>
       <c r="C258" t="inlineStr">
         <is>
-          <t>Bajaj KOM 89H</t>
+          <t>Bajaj UYL 39H</t>
         </is>
       </c>
       <c r="D258" t="inlineStr">
         <is>
-          <t>KOM89H</t>
+          <t>UYL39H</t>
         </is>
       </c>
       <c r="H258" t="n">
@@ -9584,17 +9584,17 @@
       </c>
       <c r="B259" t="inlineStr">
         <is>
-          <t>Luis Gabriel Polo</t>
+          <t>Engelo Junior</t>
         </is>
       </c>
       <c r="C259" t="inlineStr">
         <is>
-          <t>Bajaj KOM 89H</t>
+          <t>Bajaj UYL 39H</t>
         </is>
       </c>
       <c r="D259" t="inlineStr">
         <is>
-          <t>KOM89H</t>
+          <t>UYL39H</t>
         </is>
       </c>
       <c r="H259" t="n">
@@ -9615,17 +9615,17 @@
       </c>
       <c r="B260" t="inlineStr">
         <is>
-          <t>Luis Gabriel Polo</t>
+          <t>Engelo Junior</t>
         </is>
       </c>
       <c r="C260" t="inlineStr">
         <is>
-          <t>Bajaj KOM 89H</t>
+          <t>Bajaj UYL 39H</t>
         </is>
       </c>
       <c r="D260" t="inlineStr">
         <is>
-          <t>KOM89H</t>
+          <t>UYL39H</t>
         </is>
       </c>
       <c r="H260" t="n">
@@ -9646,17 +9646,17 @@
       </c>
       <c r="B261" t="inlineStr">
         <is>
-          <t>Luis Gabriel Polo</t>
+          <t>Engelo Junior</t>
         </is>
       </c>
       <c r="C261" t="inlineStr">
         <is>
-          <t>Bajaj KOM 89H</t>
+          <t>Bajaj UYL 39H</t>
         </is>
       </c>
       <c r="D261" t="inlineStr">
         <is>
-          <t>KOM89H</t>
+          <t>UYL39H</t>
         </is>
       </c>
       <c r="H261" t="n">
@@ -9677,17 +9677,17 @@
       </c>
       <c r="B262" t="inlineStr">
         <is>
-          <t>Luis Gabriel Polo</t>
+          <t>Engelo Junior</t>
         </is>
       </c>
       <c r="C262" t="inlineStr">
         <is>
-          <t>Bajaj KOM 89H</t>
+          <t>Bajaj UYL 39H</t>
         </is>
       </c>
       <c r="D262" t="inlineStr">
         <is>
-          <t>KOM89H</t>
+          <t>UYL39H</t>
         </is>
       </c>
       <c r="H262" t="n">
@@ -9708,17 +9708,17 @@
       </c>
       <c r="B263" t="inlineStr">
         <is>
-          <t>Luis Gabriel Polo</t>
+          <t>Engelo Junior</t>
         </is>
       </c>
       <c r="C263" t="inlineStr">
         <is>
-          <t>Bajaj KOM 89H</t>
+          <t>Bajaj UYL 39H</t>
         </is>
       </c>
       <c r="D263" t="inlineStr">
         <is>
-          <t>KOM89H</t>
+          <t>UYL39H</t>
         </is>
       </c>
       <c r="H263" t="n">
@@ -9739,17 +9739,17 @@
       </c>
       <c r="B264" t="inlineStr">
         <is>
-          <t>Luis Gabriel Polo</t>
+          <t>Engelo Junior</t>
         </is>
       </c>
       <c r="C264" t="inlineStr">
         <is>
-          <t>Bajaj KOM 89H</t>
+          <t>Bajaj UYL 39H</t>
         </is>
       </c>
       <c r="D264" t="inlineStr">
         <is>
-          <t>KOM89H</t>
+          <t>UYL39H</t>
         </is>
       </c>
       <c r="H264" t="n">
@@ -9770,17 +9770,17 @@
       </c>
       <c r="B265" t="inlineStr">
         <is>
-          <t>Luis Gabriel Polo</t>
+          <t>Engelo Junior</t>
         </is>
       </c>
       <c r="C265" t="inlineStr">
         <is>
-          <t>Bajaj KOM 89H</t>
+          <t>Bajaj UYL 39H</t>
         </is>
       </c>
       <c r="D265" t="inlineStr">
         <is>
-          <t>KOM89H</t>
+          <t>UYL39H</t>
         </is>
       </c>
       <c r="H265" t="n">
@@ -9801,17 +9801,17 @@
       </c>
       <c r="B266" t="inlineStr">
         <is>
-          <t>Luis Gabriel Polo</t>
+          <t>Engelo Junior</t>
         </is>
       </c>
       <c r="C266" t="inlineStr">
         <is>
-          <t>Bajaj KOM 89H</t>
+          <t>Bajaj UYL 39H</t>
         </is>
       </c>
       <c r="D266" t="inlineStr">
         <is>
-          <t>KOM89H</t>
+          <t>UYL39H</t>
         </is>
       </c>
       <c r="H266" t="n">
@@ -9832,17 +9832,17 @@
       </c>
       <c r="B267" t="inlineStr">
         <is>
-          <t>Luis Gabriel Polo</t>
+          <t>Engelo Junior</t>
         </is>
       </c>
       <c r="C267" t="inlineStr">
         <is>
-          <t>Bajaj KOM 89H</t>
+          <t>Bajaj UYL 39H</t>
         </is>
       </c>
       <c r="D267" t="inlineStr">
         <is>
-          <t>KOM89H</t>
+          <t>UYL39H</t>
         </is>
       </c>
       <c r="H267" t="n">
@@ -22108,7 +22108,7 @@
       </c>
       <c r="B663" t="inlineStr">
         <is>
-          <t>Nabro Maria Jesse</t>
+          <t>Negro Maria Jose</t>
         </is>
       </c>
       <c r="C663" t="inlineStr">
@@ -22139,7 +22139,7 @@
       </c>
       <c r="B664" t="inlineStr">
         <is>
-          <t>Nabro Maria Jesse</t>
+          <t>Negro Maria Jose</t>
         </is>
       </c>
       <c r="C664" t="inlineStr">
@@ -22170,7 +22170,7 @@
       </c>
       <c r="B665" t="inlineStr">
         <is>
-          <t>Nabro Maria Jesse</t>
+          <t>Negro Maria Jose</t>
         </is>
       </c>
       <c r="C665" t="inlineStr">
@@ -22201,7 +22201,7 @@
       </c>
       <c r="B666" t="inlineStr">
         <is>
-          <t>Nabro Maria Jesse</t>
+          <t>Negro Maria Jose</t>
         </is>
       </c>
       <c r="C666" t="inlineStr">
@@ -22232,7 +22232,7 @@
       </c>
       <c r="B667" t="inlineStr">
         <is>
-          <t>Nabro Maria Jesse</t>
+          <t>Negro Maria Jose</t>
         </is>
       </c>
       <c r="C667" t="inlineStr">
@@ -22263,7 +22263,7 @@
       </c>
       <c r="B668" t="inlineStr">
         <is>
-          <t>Nabro Maria Jesse</t>
+          <t>Negro Maria Jose</t>
         </is>
       </c>
       <c r="C668" t="inlineStr">
@@ -22294,7 +22294,7 @@
       </c>
       <c r="B669" t="inlineStr">
         <is>
-          <t>Nabro Maria Jesse</t>
+          <t>Negro Maria Jose</t>
         </is>
       </c>
       <c r="C669" t="inlineStr">
@@ -22325,7 +22325,7 @@
       </c>
       <c r="B670" t="inlineStr">
         <is>
-          <t>Nabro Maria Jesse</t>
+          <t>Negro Maria Jose</t>
         </is>
       </c>
       <c r="C670" t="inlineStr">
@@ -22356,7 +22356,7 @@
       </c>
       <c r="B671" t="inlineStr">
         <is>
-          <t>Nabro Maria Jesse</t>
+          <t>Negro Maria Jose</t>
         </is>
       </c>
       <c r="C671" t="inlineStr">
@@ -22387,7 +22387,7 @@
       </c>
       <c r="B672" t="inlineStr">
         <is>
-          <t>Nabro Maria Jesse</t>
+          <t>Negro Maria Jose</t>
         </is>
       </c>
       <c r="C672" t="inlineStr">
@@ -22418,7 +22418,7 @@
       </c>
       <c r="B673" t="inlineStr">
         <is>
-          <t>Nabro Maria Jesse</t>
+          <t>Negro Maria Jose</t>
         </is>
       </c>
       <c r="C673" t="inlineStr">
@@ -22449,7 +22449,7 @@
       </c>
       <c r="B674" t="inlineStr">
         <is>
-          <t>Nabro Maria Jesse</t>
+          <t>Negro Maria Jose</t>
         </is>
       </c>
       <c r="C674" t="inlineStr">
@@ -22480,7 +22480,7 @@
       </c>
       <c r="B675" t="inlineStr">
         <is>
-          <t>Nabro Maria Jesse</t>
+          <t>Negro Maria Jose</t>
         </is>
       </c>
       <c r="C675" t="inlineStr">
@@ -22511,7 +22511,7 @@
       </c>
       <c r="B676" t="inlineStr">
         <is>
-          <t>Nabro Maria Jesse</t>
+          <t>Negro Maria Jose</t>
         </is>
       </c>
       <c r="C676" t="inlineStr">
@@ -22542,7 +22542,7 @@
       </c>
       <c r="B677" t="inlineStr">
         <is>
-          <t>Nabro Maria Jesse</t>
+          <t>Negro Maria Jose</t>
         </is>
       </c>
       <c r="C677" t="inlineStr">
@@ -22573,7 +22573,7 @@
       </c>
       <c r="B678" t="inlineStr">
         <is>
-          <t>Nabro Maria Jesse</t>
+          <t>Negro Maria Jose</t>
         </is>
       </c>
       <c r="C678" t="inlineStr">
@@ -22604,7 +22604,7 @@
       </c>
       <c r="B679" t="inlineStr">
         <is>
-          <t>Nabro Maria Jesse</t>
+          <t>Negro Maria Jose</t>
         </is>
       </c>
       <c r="C679" t="inlineStr">
@@ -22635,7 +22635,7 @@
       </c>
       <c r="B680" t="inlineStr">
         <is>
-          <t>Nabro Maria Jesse</t>
+          <t>Negro Maria Jose</t>
         </is>
       </c>
       <c r="C680" t="inlineStr">
@@ -22666,7 +22666,7 @@
       </c>
       <c r="B681" t="inlineStr">
         <is>
-          <t>Nabro Maria Jesse</t>
+          <t>Negro Maria Jose</t>
         </is>
       </c>
       <c r="C681" t="inlineStr">
@@ -22697,7 +22697,7 @@
       </c>
       <c r="B682" t="inlineStr">
         <is>
-          <t>Nabro Maria Jesse</t>
+          <t>Negro Maria Jose</t>
         </is>
       </c>
       <c r="C682" t="inlineStr">
@@ -22728,7 +22728,7 @@
       </c>
       <c r="B683" t="inlineStr">
         <is>
-          <t>Nabro Maria Jesse</t>
+          <t>Negro Maria Jose</t>
         </is>
       </c>
       <c r="C683" t="inlineStr">
@@ -22759,7 +22759,7 @@
       </c>
       <c r="B684" t="inlineStr">
         <is>
-          <t>Nabro Maria Jesse</t>
+          <t>Negro Maria Jose</t>
         </is>
       </c>
       <c r="C684" t="inlineStr">
@@ -22790,7 +22790,7 @@
       </c>
       <c r="B685" t="inlineStr">
         <is>
-          <t>Nabro Maria Jesse</t>
+          <t>Negro Maria Jose</t>
         </is>
       </c>
       <c r="C685" t="inlineStr">
@@ -22821,7 +22821,7 @@
       </c>
       <c r="B686" t="inlineStr">
         <is>
-          <t>Nabro Maria Jesse</t>
+          <t>Negro Maria Jose</t>
         </is>
       </c>
       <c r="C686" t="inlineStr">
@@ -22852,7 +22852,7 @@
       </c>
       <c r="B687" t="inlineStr">
         <is>
-          <t>Nabro Maria Jesse</t>
+          <t>Negro Maria Jose</t>
         </is>
       </c>
       <c r="C687" t="inlineStr">
@@ -22883,7 +22883,7 @@
       </c>
       <c r="B688" t="inlineStr">
         <is>
-          <t>Nabro Maria Jesse</t>
+          <t>Negro Maria Jose</t>
         </is>
       </c>
       <c r="C688" t="inlineStr">
@@ -22914,7 +22914,7 @@
       </c>
       <c r="B689" t="inlineStr">
         <is>
-          <t>Nabro Maria Jesse</t>
+          <t>Negro Maria Jose</t>
         </is>
       </c>
       <c r="C689" t="inlineStr">
@@ -22945,7 +22945,7 @@
       </c>
       <c r="B690" t="inlineStr">
         <is>
-          <t>Nabro Maria Jesse</t>
+          <t>Negro Maria Jose</t>
         </is>
       </c>
       <c r="C690" t="inlineStr">
@@ -22976,7 +22976,7 @@
       </c>
       <c r="B691" t="inlineStr">
         <is>
-          <t>Nabro Maria Jesse</t>
+          <t>Negro Maria Jose</t>
         </is>
       </c>
       <c r="C691" t="inlineStr">
@@ -23007,7 +23007,7 @@
       </c>
       <c r="B692" t="inlineStr">
         <is>
-          <t>Nabro Maria Jesse</t>
+          <t>Negro Maria Jose</t>
         </is>
       </c>
       <c r="C692" t="inlineStr">
@@ -23038,7 +23038,7 @@
       </c>
       <c r="B693" t="inlineStr">
         <is>
-          <t>Nabro Maria Jesse</t>
+          <t>Negro Maria Jose</t>
         </is>
       </c>
       <c r="C693" t="inlineStr">
@@ -23069,7 +23069,7 @@
       </c>
       <c r="B694" t="inlineStr">
         <is>
-          <t>Nabro Maria Jesse</t>
+          <t>Negro Maria Jose</t>
         </is>
       </c>
       <c r="C694" t="inlineStr">
@@ -23100,7 +23100,7 @@
       </c>
       <c r="B695" t="inlineStr">
         <is>
-          <t>Nabro Maria Jesse</t>
+          <t>Negro Maria Jose</t>
         </is>
       </c>
       <c r="C695" t="inlineStr">
@@ -23131,7 +23131,7 @@
       </c>
       <c r="B696" t="inlineStr">
         <is>
-          <t>Nabro Maria Jesse</t>
+          <t>Negro Maria Jose</t>
         </is>
       </c>
       <c r="C696" t="inlineStr">
@@ -23162,7 +23162,7 @@
       </c>
       <c r="B697" t="inlineStr">
         <is>
-          <t>Nabro Maria Jesse</t>
+          <t>Negro Maria Jose</t>
         </is>
       </c>
       <c r="C697" t="inlineStr">
@@ -23193,7 +23193,7 @@
       </c>
       <c r="B698" t="inlineStr">
         <is>
-          <t>Nabro Maria Jesse</t>
+          <t>Negro Maria Jose</t>
         </is>
       </c>
       <c r="C698" t="inlineStr">
@@ -23224,7 +23224,7 @@
       </c>
       <c r="B699" t="inlineStr">
         <is>
-          <t>Nabro Maria Jesse</t>
+          <t>Negro Maria Jose</t>
         </is>
       </c>
       <c r="C699" t="inlineStr">
@@ -23255,7 +23255,7 @@
       </c>
       <c r="B700" t="inlineStr">
         <is>
-          <t>Nabro Maria Jesse</t>
+          <t>Negro Maria Jose</t>
         </is>
       </c>
       <c r="C700" t="inlineStr">
@@ -23286,7 +23286,7 @@
       </c>
       <c r="B701" t="inlineStr">
         <is>
-          <t>Nabro Maria Jesse</t>
+          <t>Negro Maria Jose</t>
         </is>
       </c>
       <c r="C701" t="inlineStr">
@@ -23317,7 +23317,7 @@
       </c>
       <c r="B702" t="inlineStr">
         <is>
-          <t>Nabro Maria Jesse</t>
+          <t>Negro Maria Jose</t>
         </is>
       </c>
       <c r="C702" t="inlineStr">
@@ -23348,7 +23348,7 @@
       </c>
       <c r="B703" t="inlineStr">
         <is>
-          <t>Nabro Maria Jesse</t>
+          <t>Negro Maria Jose</t>
         </is>
       </c>
       <c r="C703" t="inlineStr">
@@ -23379,7 +23379,7 @@
       </c>
       <c r="B704" t="inlineStr">
         <is>
-          <t>Nabro Maria Jesse</t>
+          <t>Negro Maria Jose</t>
         </is>
       </c>
       <c r="C704" t="inlineStr">
@@ -23410,7 +23410,7 @@
       </c>
       <c r="B705" t="inlineStr">
         <is>
-          <t>Nabro Maria Jesse</t>
+          <t>Negro Maria Jose</t>
         </is>
       </c>
       <c r="C705" t="inlineStr">
@@ -23441,7 +23441,7 @@
       </c>
       <c r="B706" t="inlineStr">
         <is>
-          <t>Nabro Maria Jesse</t>
+          <t>Negro Maria Jose</t>
         </is>
       </c>
       <c r="C706" t="inlineStr">
@@ -23472,7 +23472,7 @@
       </c>
       <c r="B707" t="inlineStr">
         <is>
-          <t>Nabro Maria Jesse</t>
+          <t>Negro Maria Jose</t>
         </is>
       </c>
       <c r="C707" t="inlineStr">
@@ -23503,7 +23503,7 @@
       </c>
       <c r="B708" t="inlineStr">
         <is>
-          <t>Nabro Maria Jesse</t>
+          <t>Negro Maria Jose</t>
         </is>
       </c>
       <c r="C708" t="inlineStr">
@@ -23534,7 +23534,7 @@
       </c>
       <c r="B709" t="inlineStr">
         <is>
-          <t>Nabro Maria Jesse</t>
+          <t>Negro Maria Jose</t>
         </is>
       </c>
       <c r="C709" t="inlineStr">
@@ -23565,7 +23565,7 @@
       </c>
       <c r="B710" t="inlineStr">
         <is>
-          <t>Nabro Maria Jesse</t>
+          <t>Negro Maria Jose</t>
         </is>
       </c>
       <c r="C710" t="inlineStr">
@@ -23596,7 +23596,7 @@
       </c>
       <c r="B711" t="inlineStr">
         <is>
-          <t>Nabro Maria Jesse</t>
+          <t>Negro Maria Jose</t>
         </is>
       </c>
       <c r="C711" t="inlineStr">
@@ -23627,7 +23627,7 @@
       </c>
       <c r="B712" t="inlineStr">
         <is>
-          <t>Nabro Maria Jesse</t>
+          <t>Negro Maria Jose</t>
         </is>
       </c>
       <c r="C712" t="inlineStr">
@@ -23658,7 +23658,7 @@
       </c>
       <c r="B713" t="inlineStr">
         <is>
-          <t>Nabro Maria Jesse</t>
+          <t>Negro Maria Jose</t>
         </is>
       </c>
       <c r="C713" t="inlineStr">
@@ -23689,7 +23689,7 @@
       </c>
       <c r="B714" t="inlineStr">
         <is>
-          <t>Luis Katherin Estor</t>
+          <t>Sr Pedro</t>
         </is>
       </c>
       <c r="C714" t="inlineStr">
@@ -23720,7 +23720,7 @@
       </c>
       <c r="B715" t="inlineStr">
         <is>
-          <t>Luis Katherin Estor</t>
+          <t>Sr Pedro</t>
         </is>
       </c>
       <c r="C715" t="inlineStr">
@@ -23751,7 +23751,7 @@
       </c>
       <c r="B716" t="inlineStr">
         <is>
-          <t>Luis Katherin Estor</t>
+          <t>Sr Pedro</t>
         </is>
       </c>
       <c r="C716" t="inlineStr">
@@ -23782,7 +23782,7 @@
       </c>
       <c r="B717" t="inlineStr">
         <is>
-          <t>Luis Katherin Estor</t>
+          <t>Sr Pedro</t>
         </is>
       </c>
       <c r="C717" t="inlineStr">
@@ -23813,7 +23813,7 @@
       </c>
       <c r="B718" t="inlineStr">
         <is>
-          <t>Luis Katherin Estor</t>
+          <t>Sr Pedro</t>
         </is>
       </c>
       <c r="C718" t="inlineStr">
@@ -23844,7 +23844,7 @@
       </c>
       <c r="B719" t="inlineStr">
         <is>
-          <t>Luis Katherin Estor</t>
+          <t>Sr Pedro</t>
         </is>
       </c>
       <c r="C719" t="inlineStr">
@@ -23875,7 +23875,7 @@
       </c>
       <c r="B720" t="inlineStr">
         <is>
-          <t>Luis Katherin Estor</t>
+          <t>Sr Pedro</t>
         </is>
       </c>
       <c r="C720" t="inlineStr">
@@ -23906,7 +23906,7 @@
       </c>
       <c r="B721" t="inlineStr">
         <is>
-          <t>Luis Katherin Estor</t>
+          <t>Sr Pedro</t>
         </is>
       </c>
       <c r="C721" t="inlineStr">
@@ -23937,7 +23937,7 @@
       </c>
       <c r="B722" t="inlineStr">
         <is>
-          <t>Luis Katherin Estor</t>
+          <t>Sr Pedro</t>
         </is>
       </c>
       <c r="C722" t="inlineStr">
@@ -23968,7 +23968,7 @@
       </c>
       <c r="B723" t="inlineStr">
         <is>
-          <t>Luis Katherin Estor</t>
+          <t>Sr Pedro</t>
         </is>
       </c>
       <c r="C723" t="inlineStr">
@@ -23999,7 +23999,7 @@
       </c>
       <c r="B724" t="inlineStr">
         <is>
-          <t>Luis Katherin Estor</t>
+          <t>Sr Pedro</t>
         </is>
       </c>
       <c r="C724" t="inlineStr">
@@ -24030,7 +24030,7 @@
       </c>
       <c r="B725" t="inlineStr">
         <is>
-          <t>Luis Katherin Estor</t>
+          <t>Sr Pedro</t>
         </is>
       </c>
       <c r="C725" t="inlineStr">
@@ -24061,7 +24061,7 @@
       </c>
       <c r="B726" t="inlineStr">
         <is>
-          <t>Luis Katherin Estor</t>
+          <t>Sr Pedro</t>
         </is>
       </c>
       <c r="C726" t="inlineStr">
@@ -24092,7 +24092,7 @@
       </c>
       <c r="B727" t="inlineStr">
         <is>
-          <t>Luis Katherin Estor</t>
+          <t>Sr Pedro</t>
         </is>
       </c>
       <c r="C727" t="inlineStr">
@@ -24123,7 +24123,7 @@
       </c>
       <c r="B728" t="inlineStr">
         <is>
-          <t>Luis Katherin Estor</t>
+          <t>Sr Pedro</t>
         </is>
       </c>
       <c r="C728" t="inlineStr">
@@ -24154,7 +24154,7 @@
       </c>
       <c r="B729" t="inlineStr">
         <is>
-          <t>Luis Katherin Estor</t>
+          <t>Sr Pedro</t>
         </is>
       </c>
       <c r="C729" t="inlineStr">
@@ -24185,7 +24185,7 @@
       </c>
       <c r="B730" t="inlineStr">
         <is>
-          <t>Luis Katherin Estor</t>
+          <t>Sr Pedro</t>
         </is>
       </c>
       <c r="C730" t="inlineStr">
@@ -24216,7 +24216,7 @@
       </c>
       <c r="B731" t="inlineStr">
         <is>
-          <t>Luis Katherin Estor</t>
+          <t>Sr Pedro</t>
         </is>
       </c>
       <c r="C731" t="inlineStr">
@@ -24247,7 +24247,7 @@
       </c>
       <c r="B732" t="inlineStr">
         <is>
-          <t>Luis Katherin Estor</t>
+          <t>Sr Pedro</t>
         </is>
       </c>
       <c r="C732" t="inlineStr">
@@ -24278,7 +24278,7 @@
       </c>
       <c r="B733" t="inlineStr">
         <is>
-          <t>Luis Katherin Estor</t>
+          <t>Sr Pedro</t>
         </is>
       </c>
       <c r="C733" t="inlineStr">
@@ -24309,7 +24309,7 @@
       </c>
       <c r="B734" t="inlineStr">
         <is>
-          <t>Luis Katherin Estor</t>
+          <t>Sr Pedro</t>
         </is>
       </c>
       <c r="C734" t="inlineStr">
@@ -24340,7 +24340,7 @@
       </c>
       <c r="B735" t="inlineStr">
         <is>
-          <t>Luis Katherin Estor</t>
+          <t>Sr Pedro</t>
         </is>
       </c>
       <c r="C735" t="inlineStr">
@@ -24371,7 +24371,7 @@
       </c>
       <c r="B736" t="inlineStr">
         <is>
-          <t>Luis Katherin Estor</t>
+          <t>Sr Pedro</t>
         </is>
       </c>
       <c r="C736" t="inlineStr">
@@ -24402,7 +24402,7 @@
       </c>
       <c r="B737" t="inlineStr">
         <is>
-          <t>Luis Katherin Estor</t>
+          <t>Sr Pedro</t>
         </is>
       </c>
       <c r="C737" t="inlineStr">
@@ -24433,7 +24433,7 @@
       </c>
       <c r="B738" t="inlineStr">
         <is>
-          <t>Luis Katherin Estor</t>
+          <t>Sr Pedro</t>
         </is>
       </c>
       <c r="C738" t="inlineStr">
@@ -24464,7 +24464,7 @@
       </c>
       <c r="B739" t="inlineStr">
         <is>
-          <t>Luis Katherin Estor</t>
+          <t>Sr Pedro</t>
         </is>
       </c>
       <c r="C739" t="inlineStr">
@@ -24495,7 +24495,7 @@
       </c>
       <c r="B740" t="inlineStr">
         <is>
-          <t>Luis Katherin Estor</t>
+          <t>Sr Pedro</t>
         </is>
       </c>
       <c r="C740" t="inlineStr">
@@ -24526,7 +24526,7 @@
       </c>
       <c r="B741" t="inlineStr">
         <is>
-          <t>Luis Katherin Estor</t>
+          <t>Sr Pedro</t>
         </is>
       </c>
       <c r="C741" t="inlineStr">
@@ -24557,7 +24557,7 @@
       </c>
       <c r="B742" t="inlineStr">
         <is>
-          <t>Luis Katherin Estor</t>
+          <t>Sr Pedro</t>
         </is>
       </c>
       <c r="C742" t="inlineStr">
@@ -24588,7 +24588,7 @@
       </c>
       <c r="B743" t="inlineStr">
         <is>
-          <t>Luis Katherin Estor</t>
+          <t>Sr Pedro</t>
         </is>
       </c>
       <c r="C743" t="inlineStr">
@@ -24619,7 +24619,7 @@
       </c>
       <c r="B744" t="inlineStr">
         <is>
-          <t>Luis Katherin Estor</t>
+          <t>Sr Pedro</t>
         </is>
       </c>
       <c r="C744" t="inlineStr">
@@ -24650,7 +24650,7 @@
       </c>
       <c r="B745" t="inlineStr">
         <is>
-          <t>Luis Katherin Estor</t>
+          <t>Sr Pedro</t>
         </is>
       </c>
       <c r="C745" t="inlineStr">
@@ -24681,7 +24681,7 @@
       </c>
       <c r="B746" t="inlineStr">
         <is>
-          <t>Luis Katherin Estor</t>
+          <t>Sr Pedro</t>
         </is>
       </c>
       <c r="C746" t="inlineStr">
@@ -24712,7 +24712,7 @@
       </c>
       <c r="B747" t="inlineStr">
         <is>
-          <t>Luis Katherin Estor</t>
+          <t>Sr Pedro</t>
         </is>
       </c>
       <c r="C747" t="inlineStr">
@@ -24743,7 +24743,7 @@
       </c>
       <c r="B748" t="inlineStr">
         <is>
-          <t>Luis Katherin Estor</t>
+          <t>Sr Pedro</t>
         </is>
       </c>
       <c r="C748" t="inlineStr">
@@ -24774,7 +24774,7 @@
       </c>
       <c r="B749" t="inlineStr">
         <is>
-          <t>Luis Katherin Estor</t>
+          <t>Sr Pedro</t>
         </is>
       </c>
       <c r="C749" t="inlineStr">
@@ -24805,7 +24805,7 @@
       </c>
       <c r="B750" t="inlineStr">
         <is>
-          <t>Luis Katherin Estor</t>
+          <t>Sr Pedro</t>
         </is>
       </c>
       <c r="C750" t="inlineStr">
@@ -24836,7 +24836,7 @@
       </c>
       <c r="B751" t="inlineStr">
         <is>
-          <t>Luis Katherin Estor</t>
+          <t>Sr Pedro</t>
         </is>
       </c>
       <c r="C751" t="inlineStr">
@@ -24867,7 +24867,7 @@
       </c>
       <c r="B752" t="inlineStr">
         <is>
-          <t>Luis Katherin Estor</t>
+          <t>Sr Pedro</t>
         </is>
       </c>
       <c r="C752" t="inlineStr">
@@ -24898,7 +24898,7 @@
       </c>
       <c r="B753" t="inlineStr">
         <is>
-          <t>Luis Katherin Estor</t>
+          <t>Sr Pedro</t>
         </is>
       </c>
       <c r="C753" t="inlineStr">
@@ -24929,7 +24929,7 @@
       </c>
       <c r="B754" t="inlineStr">
         <is>
-          <t>Luis Katherin Estor</t>
+          <t>Sr Pedro</t>
         </is>
       </c>
       <c r="C754" t="inlineStr">
@@ -24960,7 +24960,7 @@
       </c>
       <c r="B755" t="inlineStr">
         <is>
-          <t>Luis Katherin Estor</t>
+          <t>Sr Pedro</t>
         </is>
       </c>
       <c r="C755" t="inlineStr">
@@ -24991,7 +24991,7 @@
       </c>
       <c r="B756" t="inlineStr">
         <is>
-          <t>Luis Katherin Estor</t>
+          <t>Sr Pedro</t>
         </is>
       </c>
       <c r="C756" t="inlineStr">
@@ -25022,7 +25022,7 @@
       </c>
       <c r="B757" t="inlineStr">
         <is>
-          <t>Luis Katherin Estor</t>
+          <t>Sr Pedro</t>
         </is>
       </c>
       <c r="C757" t="inlineStr">
@@ -25053,7 +25053,7 @@
       </c>
       <c r="B758" t="inlineStr">
         <is>
-          <t>Luis Katherin Estor</t>
+          <t>Sr Pedro</t>
         </is>
       </c>
       <c r="C758" t="inlineStr">
@@ -25084,7 +25084,7 @@
       </c>
       <c r="B759" t="inlineStr">
         <is>
-          <t>Luis Katherin Estor</t>
+          <t>Sr Pedro</t>
         </is>
       </c>
       <c r="C759" t="inlineStr">
@@ -25115,7 +25115,7 @@
       </c>
       <c r="B760" t="inlineStr">
         <is>
-          <t>Luis Katherin Estor</t>
+          <t>Sr Pedro</t>
         </is>
       </c>
       <c r="C760" t="inlineStr">
@@ -25146,7 +25146,7 @@
       </c>
       <c r="B761" t="inlineStr">
         <is>
-          <t>Luis Katherin Estor</t>
+          <t>Sr Pedro</t>
         </is>
       </c>
       <c r="C761" t="inlineStr">
@@ -25177,7 +25177,7 @@
       </c>
       <c r="B762" t="inlineStr">
         <is>
-          <t>Luis Katherin Estor</t>
+          <t>Sr Pedro</t>
         </is>
       </c>
       <c r="C762" t="inlineStr">
@@ -25208,7 +25208,7 @@
       </c>
       <c r="B763" t="inlineStr">
         <is>
-          <t>Luis Katherin Estor</t>
+          <t>Sr Pedro</t>
         </is>
       </c>
       <c r="C763" t="inlineStr">
@@ -25239,7 +25239,7 @@
       </c>
       <c r="B764" t="inlineStr">
         <is>
-          <t>Luis Katherin Estor</t>
+          <t>Sr Pedro</t>
         </is>
       </c>
       <c r="C764" t="inlineStr">
@@ -25270,7 +25270,7 @@
       </c>
       <c r="B765" t="inlineStr">
         <is>
-          <t>Luis Katherin Estor</t>
+          <t>Sr Pedro</t>
         </is>
       </c>
       <c r="C765" t="inlineStr">
@@ -25301,7 +25301,7 @@
       </c>
       <c r="B766" t="inlineStr">
         <is>
-          <t>Luis Katherin Estor</t>
+          <t>Sr Pedro</t>
         </is>
       </c>
       <c r="C766" t="inlineStr">
@@ -25332,7 +25332,7 @@
       </c>
       <c r="B767" t="inlineStr">
         <is>
-          <t>Luis Katherin Estor</t>
+          <t>Sr Pedro</t>
         </is>
       </c>
       <c r="C767" t="inlineStr">
@@ -28277,7 +28277,7 @@
       </c>
       <c r="B862" t="inlineStr">
         <is>
-          <t>Braillon</t>
+          <t>Brayan</t>
         </is>
       </c>
       <c r="C862" t="inlineStr">
@@ -28308,7 +28308,7 @@
       </c>
       <c r="B863" t="inlineStr">
         <is>
-          <t>Braillon</t>
+          <t>Brayan</t>
         </is>
       </c>
       <c r="C863" t="inlineStr">
@@ -28339,7 +28339,7 @@
       </c>
       <c r="B864" t="inlineStr">
         <is>
-          <t>Braillon</t>
+          <t>Brayan</t>
         </is>
       </c>
       <c r="C864" t="inlineStr">
@@ -28370,7 +28370,7 @@
       </c>
       <c r="B865" t="inlineStr">
         <is>
-          <t>Braillon</t>
+          <t>Brayan</t>
         </is>
       </c>
       <c r="C865" t="inlineStr">
@@ -28401,7 +28401,7 @@
       </c>
       <c r="B866" t="inlineStr">
         <is>
-          <t>Braillon</t>
+          <t>Brayan</t>
         </is>
       </c>
       <c r="C866" t="inlineStr">
@@ -28432,7 +28432,7 @@
       </c>
       <c r="B867" t="inlineStr">
         <is>
-          <t>Braillon</t>
+          <t>Brayan</t>
         </is>
       </c>
       <c r="C867" t="inlineStr">
@@ -28463,7 +28463,7 @@
       </c>
       <c r="B868" t="inlineStr">
         <is>
-          <t>Braillon</t>
+          <t>Brayan</t>
         </is>
       </c>
       <c r="C868" t="inlineStr">
@@ -28494,7 +28494,7 @@
       </c>
       <c r="B869" t="inlineStr">
         <is>
-          <t>Braillon</t>
+          <t>Brayan</t>
         </is>
       </c>
       <c r="C869" t="inlineStr">
@@ -28525,7 +28525,7 @@
       </c>
       <c r="B870" t="inlineStr">
         <is>
-          <t>Braillon</t>
+          <t>Brayan</t>
         </is>
       </c>
       <c r="C870" t="inlineStr">
@@ -28556,7 +28556,7 @@
       </c>
       <c r="B871" t="inlineStr">
         <is>
-          <t>Braillon</t>
+          <t>Brayan</t>
         </is>
       </c>
       <c r="C871" t="inlineStr">
@@ -28587,7 +28587,7 @@
       </c>
       <c r="B872" t="inlineStr">
         <is>
-          <t>Braillon</t>
+          <t>Brayan</t>
         </is>
       </c>
       <c r="C872" t="inlineStr">
@@ -28618,7 +28618,7 @@
       </c>
       <c r="B873" t="inlineStr">
         <is>
-          <t>Braillon</t>
+          <t>Brayan</t>
         </is>
       </c>
       <c r="C873" t="inlineStr">
@@ -28649,7 +28649,7 @@
       </c>
       <c r="B874" t="inlineStr">
         <is>
-          <t>Braillon</t>
+          <t>Brayan</t>
         </is>
       </c>
       <c r="C874" t="inlineStr">
@@ -28680,7 +28680,7 @@
       </c>
       <c r="B875" t="inlineStr">
         <is>
-          <t>Braillon</t>
+          <t>Brayan</t>
         </is>
       </c>
       <c r="C875" t="inlineStr">
@@ -28711,7 +28711,7 @@
       </c>
       <c r="B876" t="inlineStr">
         <is>
-          <t>Braillon</t>
+          <t>Brayan</t>
         </is>
       </c>
       <c r="C876" t="inlineStr">
@@ -28742,7 +28742,7 @@
       </c>
       <c r="B877" t="inlineStr">
         <is>
-          <t>Braillon</t>
+          <t>Brayan</t>
         </is>
       </c>
       <c r="C877" t="inlineStr">
@@ -28773,7 +28773,7 @@
       </c>
       <c r="B878" t="inlineStr">
         <is>
-          <t>Braillon</t>
+          <t>Brayan</t>
         </is>
       </c>
       <c r="C878" t="inlineStr">
@@ -28804,7 +28804,7 @@
       </c>
       <c r="B879" t="inlineStr">
         <is>
-          <t>Braillon</t>
+          <t>Brayan</t>
         </is>
       </c>
       <c r="C879" t="inlineStr">
@@ -28835,7 +28835,7 @@
       </c>
       <c r="B880" t="inlineStr">
         <is>
-          <t>Braillon</t>
+          <t>Brayan</t>
         </is>
       </c>
       <c r="C880" t="inlineStr">
@@ -28866,7 +28866,7 @@
       </c>
       <c r="B881" t="inlineStr">
         <is>
-          <t>Braillon</t>
+          <t>Brayan</t>
         </is>
       </c>
       <c r="C881" t="inlineStr">
@@ -28897,7 +28897,7 @@
       </c>
       <c r="B882" t="inlineStr">
         <is>
-          <t>Braillon</t>
+          <t>Brayan</t>
         </is>
       </c>
       <c r="C882" t="inlineStr">
@@ -28928,7 +28928,7 @@
       </c>
       <c r="B883" t="inlineStr">
         <is>
-          <t>Braillon</t>
+          <t>Brayan</t>
         </is>
       </c>
       <c r="C883" t="inlineStr">
@@ -28959,7 +28959,7 @@
       </c>
       <c r="B884" t="inlineStr">
         <is>
-          <t>Braillon</t>
+          <t>Brayan</t>
         </is>
       </c>
       <c r="C884" t="inlineStr">
@@ -28990,7 +28990,7 @@
       </c>
       <c r="B885" t="inlineStr">
         <is>
-          <t>Braillon</t>
+          <t>Brayan</t>
         </is>
       </c>
       <c r="C885" t="inlineStr">
@@ -29021,7 +29021,7 @@
       </c>
       <c r="B886" t="inlineStr">
         <is>
-          <t>Braillon</t>
+          <t>Brayan</t>
         </is>
       </c>
       <c r="C886" t="inlineStr">
@@ -29052,7 +29052,7 @@
       </c>
       <c r="B887" t="inlineStr">
         <is>
-          <t>Braillon</t>
+          <t>Brayan</t>
         </is>
       </c>
       <c r="C887" t="inlineStr">
@@ -29083,7 +29083,7 @@
       </c>
       <c r="B888" t="inlineStr">
         <is>
-          <t>Braillon</t>
+          <t>Brayan</t>
         </is>
       </c>
       <c r="C888" t="inlineStr">
@@ -29114,7 +29114,7 @@
       </c>
       <c r="B889" t="inlineStr">
         <is>
-          <t>Braillon</t>
+          <t>Brayan</t>
         </is>
       </c>
       <c r="C889" t="inlineStr">
@@ -29145,7 +29145,7 @@
       </c>
       <c r="B890" t="inlineStr">
         <is>
-          <t>Braillon</t>
+          <t>Brayan</t>
         </is>
       </c>
       <c r="C890" t="inlineStr">
@@ -29176,7 +29176,7 @@
       </c>
       <c r="B891" t="inlineStr">
         <is>
-          <t>Braillon</t>
+          <t>Brayan</t>
         </is>
       </c>
       <c r="C891" t="inlineStr">
@@ -29207,7 +29207,7 @@
       </c>
       <c r="B892" t="inlineStr">
         <is>
-          <t>Braillon</t>
+          <t>Brayan</t>
         </is>
       </c>
       <c r="C892" t="inlineStr">
@@ -29238,7 +29238,7 @@
       </c>
       <c r="B893" t="inlineStr">
         <is>
-          <t>Braillon</t>
+          <t>Brayan</t>
         </is>
       </c>
       <c r="C893" t="inlineStr">
@@ -29269,7 +29269,7 @@
       </c>
       <c r="B894" t="inlineStr">
         <is>
-          <t>Braillon</t>
+          <t>Brayan</t>
         </is>
       </c>
       <c r="C894" t="inlineStr">
@@ -29300,7 +29300,7 @@
       </c>
       <c r="B895" t="inlineStr">
         <is>
-          <t>Braillon</t>
+          <t>Brayan</t>
         </is>
       </c>
       <c r="C895" t="inlineStr">
@@ -29331,7 +29331,7 @@
       </c>
       <c r="B896" t="inlineStr">
         <is>
-          <t>Braillon</t>
+          <t>Brayan</t>
         </is>
       </c>
       <c r="C896" t="inlineStr">
@@ -29362,7 +29362,7 @@
       </c>
       <c r="B897" t="inlineStr">
         <is>
-          <t>Braillon</t>
+          <t>Brayan</t>
         </is>
       </c>
       <c r="C897" t="inlineStr">
@@ -29393,7 +29393,7 @@
       </c>
       <c r="B898" t="inlineStr">
         <is>
-          <t>Braillon</t>
+          <t>Brayan</t>
         </is>
       </c>
       <c r="C898" t="inlineStr">
@@ -29424,7 +29424,7 @@
       </c>
       <c r="B899" t="inlineStr">
         <is>
-          <t>Braillon</t>
+          <t>Brayan</t>
         </is>
       </c>
       <c r="C899" t="inlineStr">
@@ -29455,7 +29455,7 @@
       </c>
       <c r="B900" t="inlineStr">
         <is>
-          <t>Braillon</t>
+          <t>Brayan</t>
         </is>
       </c>
       <c r="C900" t="inlineStr">
@@ -29486,7 +29486,7 @@
       </c>
       <c r="B901" t="inlineStr">
         <is>
-          <t>Braillon</t>
+          <t>Brayan</t>
         </is>
       </c>
       <c r="C901" t="inlineStr">
@@ -29517,7 +29517,7 @@
       </c>
       <c r="B902" t="inlineStr">
         <is>
-          <t>Braillon</t>
+          <t>Brayan</t>
         </is>
       </c>
       <c r="C902" t="inlineStr">
@@ -29548,7 +29548,7 @@
       </c>
       <c r="B903" t="inlineStr">
         <is>
-          <t>Braillon</t>
+          <t>Brayan</t>
         </is>
       </c>
       <c r="C903" t="inlineStr">
@@ -29579,7 +29579,7 @@
       </c>
       <c r="B904" t="inlineStr">
         <is>
-          <t>Braillon</t>
+          <t>Brayan</t>
         </is>
       </c>
       <c r="C904" t="inlineStr">
@@ -31718,7 +31718,7 @@
       </c>
       <c r="B973" t="inlineStr">
         <is>
-          <t>Erzik</t>
+          <t>Erik</t>
         </is>
       </c>
       <c r="C973" t="inlineStr">
@@ -31749,7 +31749,7 @@
       </c>
       <c r="B974" t="inlineStr">
         <is>
-          <t>Erzik</t>
+          <t>Erik</t>
         </is>
       </c>
       <c r="C974" t="inlineStr">
@@ -31780,7 +31780,7 @@
       </c>
       <c r="B975" t="inlineStr">
         <is>
-          <t>Erzik</t>
+          <t>Erik</t>
         </is>
       </c>
       <c r="C975" t="inlineStr">
@@ -31811,7 +31811,7 @@
       </c>
       <c r="B976" t="inlineStr">
         <is>
-          <t>Erzik</t>
+          <t>Erik</t>
         </is>
       </c>
       <c r="C976" t="inlineStr">
@@ -31842,7 +31842,7 @@
       </c>
       <c r="B977" t="inlineStr">
         <is>
-          <t>Erzik</t>
+          <t>Erik</t>
         </is>
       </c>
       <c r="C977" t="inlineStr">
@@ -31873,7 +31873,7 @@
       </c>
       <c r="B978" t="inlineStr">
         <is>
-          <t>Erzik</t>
+          <t>Erik</t>
         </is>
       </c>
       <c r="C978" t="inlineStr">
@@ -31904,7 +31904,7 @@
       </c>
       <c r="B979" t="inlineStr">
         <is>
-          <t>Erzik</t>
+          <t>Erik</t>
         </is>
       </c>
       <c r="C979" t="inlineStr">
@@ -31935,7 +31935,7 @@
       </c>
       <c r="B980" t="inlineStr">
         <is>
-          <t>Erzik</t>
+          <t>Erik</t>
         </is>
       </c>
       <c r="C980" t="inlineStr">
@@ -31966,7 +31966,7 @@
       </c>
       <c r="B981" t="inlineStr">
         <is>
-          <t>Erzik</t>
+          <t>Erik</t>
         </is>
       </c>
       <c r="C981" t="inlineStr">
@@ -31997,7 +31997,7 @@
       </c>
       <c r="B982" t="inlineStr">
         <is>
-          <t>Erzik</t>
+          <t>Erik</t>
         </is>
       </c>
       <c r="C982" t="inlineStr">
@@ -32028,7 +32028,7 @@
       </c>
       <c r="B983" t="inlineStr">
         <is>
-          <t>Erzik</t>
+          <t>Erik</t>
         </is>
       </c>
       <c r="C983" t="inlineStr">
@@ -32059,7 +32059,7 @@
       </c>
       <c r="B984" t="inlineStr">
         <is>
-          <t>Erzik</t>
+          <t>Erik</t>
         </is>
       </c>
       <c r="C984" t="inlineStr">
@@ -32090,7 +32090,7 @@
       </c>
       <c r="B985" t="inlineStr">
         <is>
-          <t>Erzik</t>
+          <t>Erik</t>
         </is>
       </c>
       <c r="C985" t="inlineStr">
@@ -32121,7 +32121,7 @@
       </c>
       <c r="B986" t="inlineStr">
         <is>
-          <t>Erzik</t>
+          <t>Erik</t>
         </is>
       </c>
       <c r="C986" t="inlineStr">
@@ -32152,7 +32152,7 @@
       </c>
       <c r="B987" t="inlineStr">
         <is>
-          <t>Erzik</t>
+          <t>Erik</t>
         </is>
       </c>
       <c r="C987" t="inlineStr">
@@ -32183,7 +32183,7 @@
       </c>
       <c r="B988" t="inlineStr">
         <is>
-          <t>Erzik</t>
+          <t>Erik</t>
         </is>
       </c>
       <c r="C988" t="inlineStr">
@@ -32214,7 +32214,7 @@
       </c>
       <c r="B989" t="inlineStr">
         <is>
-          <t>Erzik</t>
+          <t>Erik</t>
         </is>
       </c>
       <c r="C989" t="inlineStr">
@@ -32927,7 +32927,7 @@
       </c>
       <c r="B1012" t="inlineStr">
         <is>
-          <t>Gonzado Estherline</t>
+          <t>Katherine</t>
         </is>
       </c>
       <c r="C1012" t="inlineStr">
@@ -32958,7 +32958,7 @@
       </c>
       <c r="B1013" t="inlineStr">
         <is>
-          <t>Gonzado Estherline</t>
+          <t>Katherine</t>
         </is>
       </c>
       <c r="C1013" t="inlineStr">
@@ -32989,7 +32989,7 @@
       </c>
       <c r="B1014" t="inlineStr">
         <is>
-          <t>Gonzado Estherline</t>
+          <t>Katherine</t>
         </is>
       </c>
       <c r="C1014" t="inlineStr">
@@ -33020,7 +33020,7 @@
       </c>
       <c r="B1015" t="inlineStr">
         <is>
-          <t>Gonzado Estherline</t>
+          <t>Katherine</t>
         </is>
       </c>
       <c r="C1015" t="inlineStr">
@@ -33051,7 +33051,7 @@
       </c>
       <c r="B1016" t="inlineStr">
         <is>
-          <t>Gonzado Estherline</t>
+          <t>Katherine</t>
         </is>
       </c>
       <c r="C1016" t="inlineStr">
@@ -33082,7 +33082,7 @@
       </c>
       <c r="B1017" t="inlineStr">
         <is>
-          <t>Gonzado Estherline</t>
+          <t>Katherine</t>
         </is>
       </c>
       <c r="C1017" t="inlineStr">
@@ -33113,7 +33113,7 @@
       </c>
       <c r="B1018" t="inlineStr">
         <is>
-          <t>Gonzado Estherline</t>
+          <t>Katherine</t>
         </is>
       </c>
       <c r="C1018" t="inlineStr">
@@ -33144,7 +33144,7 @@
       </c>
       <c r="B1019" t="inlineStr">
         <is>
-          <t>Gonzado Estherline</t>
+          <t>Katherine</t>
         </is>
       </c>
       <c r="C1019" t="inlineStr">
@@ -33175,7 +33175,7 @@
       </c>
       <c r="B1020" t="inlineStr">
         <is>
-          <t>Gonzado Estherline</t>
+          <t>Katherine</t>
         </is>
       </c>
       <c r="C1020" t="inlineStr">
@@ -33206,7 +33206,7 @@
       </c>
       <c r="B1021" t="inlineStr">
         <is>
-          <t>Gonzado Estherline</t>
+          <t>Katherine</t>
         </is>
       </c>
       <c r="C1021" t="inlineStr">
@@ -33237,7 +33237,7 @@
       </c>
       <c r="B1022" t="inlineStr">
         <is>
-          <t>Gonzado Estherline</t>
+          <t>Katherine</t>
         </is>
       </c>
       <c r="C1022" t="inlineStr">
@@ -33268,7 +33268,7 @@
       </c>
       <c r="B1023" t="inlineStr">
         <is>
-          <t>Gonzado Estherline</t>
+          <t>Katherine</t>
         </is>
       </c>
       <c r="C1023" t="inlineStr">
@@ -33299,7 +33299,7 @@
       </c>
       <c r="B1024" t="inlineStr">
         <is>
-          <t>Gonzado Estherline</t>
+          <t>Katherine</t>
         </is>
       </c>
       <c r="C1024" t="inlineStr">
@@ -33330,7 +33330,7 @@
       </c>
       <c r="B1025" t="inlineStr">
         <is>
-          <t>Gonzado Estherline</t>
+          <t>Katherine</t>
         </is>
       </c>
       <c r="C1025" t="inlineStr">
@@ -33361,7 +33361,7 @@
       </c>
       <c r="B1026" t="inlineStr">
         <is>
-          <t>Gonzado Estherline</t>
+          <t>Katherine</t>
         </is>
       </c>
       <c r="C1026" t="inlineStr">
@@ -33392,7 +33392,7 @@
       </c>
       <c r="B1027" t="inlineStr">
         <is>
-          <t>Gonzado Estherline</t>
+          <t>Katherine</t>
         </is>
       </c>
       <c r="C1027" t="inlineStr">
@@ -33423,7 +33423,7 @@
       </c>
       <c r="B1028" t="inlineStr">
         <is>
-          <t>Gonzado Estherline</t>
+          <t>Katherine</t>
         </is>
       </c>
       <c r="C1028" t="inlineStr">
@@ -33454,7 +33454,7 @@
       </c>
       <c r="B1029" t="inlineStr">
         <is>
-          <t>Gonzado Estherline</t>
+          <t>Katherine</t>
         </is>
       </c>
       <c r="C1029" t="inlineStr">
@@ -33485,7 +33485,7 @@
       </c>
       <c r="B1030" t="inlineStr">
         <is>
-          <t>Gonzado Estherline</t>
+          <t>Katherine</t>
         </is>
       </c>
       <c r="C1030" t="inlineStr">
@@ -33516,7 +33516,7 @@
       </c>
       <c r="B1031" t="inlineStr">
         <is>
-          <t>Gonzado Estherline</t>
+          <t>Katherine</t>
         </is>
       </c>
       <c r="C1031" t="inlineStr">
@@ -33547,7 +33547,7 @@
       </c>
       <c r="B1032" t="inlineStr">
         <is>
-          <t>Gonzado Estherline</t>
+          <t>Katherine</t>
         </is>
       </c>
       <c r="C1032" t="inlineStr">
@@ -33578,7 +33578,7 @@
       </c>
       <c r="B1033" t="inlineStr">
         <is>
-          <t>Gonzado Estherline</t>
+          <t>Katherine</t>
         </is>
       </c>
       <c r="C1033" t="inlineStr">
@@ -33609,7 +33609,7 @@
       </c>
       <c r="B1034" t="inlineStr">
         <is>
-          <t>Gonzado Estherline</t>
+          <t>Katherine</t>
         </is>
       </c>
       <c r="C1034" t="inlineStr">
@@ -33640,7 +33640,7 @@
       </c>
       <c r="B1035" t="inlineStr">
         <is>
-          <t>Gonzado Estherline</t>
+          <t>Katherine</t>
         </is>
       </c>
       <c r="C1035" t="inlineStr">
@@ -33671,7 +33671,7 @@
       </c>
       <c r="B1036" t="inlineStr">
         <is>
-          <t>Gonzado Estherline</t>
+          <t>Katherine</t>
         </is>
       </c>
       <c r="C1036" t="inlineStr">
@@ -33702,7 +33702,7 @@
       </c>
       <c r="B1037" t="inlineStr">
         <is>
-          <t>Gonzado Estherline</t>
+          <t>Katherine</t>
         </is>
       </c>
       <c r="C1037" t="inlineStr">
@@ -33733,7 +33733,7 @@
       </c>
       <c r="B1038" t="inlineStr">
         <is>
-          <t>Gonzado Estherline</t>
+          <t>Katherine</t>
         </is>
       </c>
       <c r="C1038" t="inlineStr">
@@ -33764,7 +33764,7 @@
       </c>
       <c r="B1039" t="inlineStr">
         <is>
-          <t>Gonzado Estherline</t>
+          <t>Katherine</t>
         </is>
       </c>
       <c r="C1039" t="inlineStr">
@@ -33795,7 +33795,7 @@
       </c>
       <c r="B1040" t="inlineStr">
         <is>
-          <t>Gonzado Estherline</t>
+          <t>Katherine</t>
         </is>
       </c>
       <c r="C1040" t="inlineStr">
@@ -33826,7 +33826,7 @@
       </c>
       <c r="B1041" t="inlineStr">
         <is>
-          <t>Gonzado Estherline</t>
+          <t>Katherine</t>
         </is>
       </c>
       <c r="C1041" t="inlineStr">
@@ -33857,7 +33857,7 @@
       </c>
       <c r="B1042" t="inlineStr">
         <is>
-          <t>Gonzado Estherline</t>
+          <t>Katherine</t>
         </is>
       </c>
       <c r="C1042" t="inlineStr">
@@ -33888,7 +33888,7 @@
       </c>
       <c r="B1043" t="inlineStr">
         <is>
-          <t>Gonzado Estherline</t>
+          <t>Katherine</t>
         </is>
       </c>
       <c r="C1043" t="inlineStr">
@@ -33919,7 +33919,7 @@
       </c>
       <c r="B1044" t="inlineStr">
         <is>
-          <t>Gonzado Estherline</t>
+          <t>Katherine</t>
         </is>
       </c>
       <c r="C1044" t="inlineStr">
@@ -33950,7 +33950,7 @@
       </c>
       <c r="B1045" t="inlineStr">
         <is>
-          <t>Gonzado Estherline</t>
+          <t>Katherine</t>
         </is>
       </c>
       <c r="C1045" t="inlineStr">
@@ -33981,7 +33981,7 @@
       </c>
       <c r="B1046" t="inlineStr">
         <is>
-          <t>Gonzado Estherline</t>
+          <t>Katherine</t>
         </is>
       </c>
       <c r="C1046" t="inlineStr">
@@ -34012,7 +34012,7 @@
       </c>
       <c r="B1047" t="inlineStr">
         <is>
-          <t>Gonzado Estherline</t>
+          <t>Katherine</t>
         </is>
       </c>
       <c r="C1047" t="inlineStr">
@@ -34043,7 +34043,7 @@
       </c>
       <c r="B1048" t="inlineStr">
         <is>
-          <t>Gonzado Estherline</t>
+          <t>Katherine</t>
         </is>
       </c>
       <c r="C1048" t="inlineStr">
@@ -34074,7 +34074,7 @@
       </c>
       <c r="B1049" t="inlineStr">
         <is>
-          <t>Gonzado Estherline</t>
+          <t>Katherine</t>
         </is>
       </c>
       <c r="C1049" t="inlineStr">
@@ -34105,7 +34105,7 @@
       </c>
       <c r="B1050" t="inlineStr">
         <is>
-          <t>Gonzado Estherline</t>
+          <t>Katherine</t>
         </is>
       </c>
       <c r="C1050" t="inlineStr">
@@ -34136,7 +34136,7 @@
       </c>
       <c r="B1051" t="inlineStr">
         <is>
-          <t>Gonzado Estherline</t>
+          <t>Katherine</t>
         </is>
       </c>
       <c r="C1051" t="inlineStr">
@@ -34167,7 +34167,7 @@
       </c>
       <c r="B1052" t="inlineStr">
         <is>
-          <t>Gonzado Estherline</t>
+          <t>Katherine</t>
         </is>
       </c>
       <c r="C1052" t="inlineStr">
@@ -34198,7 +34198,7 @@
       </c>
       <c r="B1053" t="inlineStr">
         <is>
-          <t>Ana Milena Juan Davit</t>
+          <t>Ana Milena-Juan David</t>
         </is>
       </c>
       <c r="C1053" t="inlineStr">
@@ -34229,7 +34229,7 @@
       </c>
       <c r="B1054" t="inlineStr">
         <is>
-          <t>Ana Milena Juan Davit</t>
+          <t>Ana Milena-Juan David</t>
         </is>
       </c>
       <c r="C1054" t="inlineStr">
@@ -34260,7 +34260,7 @@
       </c>
       <c r="B1055" t="inlineStr">
         <is>
-          <t>Ana Milena Juan Davit</t>
+          <t>Ana Milena-Juan David</t>
         </is>
       </c>
       <c r="C1055" t="inlineStr">
@@ -34291,7 +34291,7 @@
       </c>
       <c r="B1056" t="inlineStr">
         <is>
-          <t>Ana Milena Juan Davit</t>
+          <t>Ana Milena-Juan David</t>
         </is>
       </c>
       <c r="C1056" t="inlineStr">
@@ -34322,7 +34322,7 @@
       </c>
       <c r="B1057" t="inlineStr">
         <is>
-          <t>Ana Milena Juan Davit</t>
+          <t>Ana Milena-Juan David</t>
         </is>
       </c>
       <c r="C1057" t="inlineStr">
@@ -34353,7 +34353,7 @@
       </c>
       <c r="B1058" t="inlineStr">
         <is>
-          <t>Ana Milena Juan Davit</t>
+          <t>Ana Milena-Juan David</t>
         </is>
       </c>
       <c r="C1058" t="inlineStr">
@@ -34384,7 +34384,7 @@
       </c>
       <c r="B1059" t="inlineStr">
         <is>
-          <t>Ana Milena Juan Davit</t>
+          <t>Ana Milena-Juan David</t>
         </is>
       </c>
       <c r="C1059" t="inlineStr">
@@ -34415,7 +34415,7 @@
       </c>
       <c r="B1060" t="inlineStr">
         <is>
-          <t>Ana Milena Juan Davit</t>
+          <t>Ana Milena-Juan David</t>
         </is>
       </c>
       <c r="C1060" t="inlineStr">
@@ -34446,7 +34446,7 @@
       </c>
       <c r="B1061" t="inlineStr">
         <is>
-          <t>Ana Milena Juan Davit</t>
+          <t>Ana Milena-Juan David</t>
         </is>
       </c>
       <c r="C1061" t="inlineStr">
@@ -34477,7 +34477,7 @@
       </c>
       <c r="B1062" t="inlineStr">
         <is>
-          <t>Ana Milena Juan Davit</t>
+          <t>Ana Milena-Juan David</t>
         </is>
       </c>
       <c r="C1062" t="inlineStr">
@@ -34508,7 +34508,7 @@
       </c>
       <c r="B1063" t="inlineStr">
         <is>
-          <t>Ana Milena Juan Davit</t>
+          <t>Ana Milena-Juan David</t>
         </is>
       </c>
       <c r="C1063" t="inlineStr">
@@ -34539,7 +34539,7 @@
       </c>
       <c r="B1064" t="inlineStr">
         <is>
-          <t>Ana Milena Juan Davit</t>
+          <t>Ana Milena-Juan David</t>
         </is>
       </c>
       <c r="C1064" t="inlineStr">
@@ -34570,7 +34570,7 @@
       </c>
       <c r="B1065" t="inlineStr">
         <is>
-          <t>Ana Milena Juan Davit</t>
+          <t>Ana Milena-Juan David</t>
         </is>
       </c>
       <c r="C1065" t="inlineStr">
@@ -34601,7 +34601,7 @@
       </c>
       <c r="B1066" t="inlineStr">
         <is>
-          <t>Ana Milena Juan Davit</t>
+          <t>Ana Milena-Juan David</t>
         </is>
       </c>
       <c r="C1066" t="inlineStr">
@@ -34632,7 +34632,7 @@
       </c>
       <c r="B1067" t="inlineStr">
         <is>
-          <t>Ana Milena Juan Davit</t>
+          <t>Ana Milena-Juan David</t>
         </is>
       </c>
       <c r="C1067" t="inlineStr">
@@ -34663,7 +34663,7 @@
       </c>
       <c r="B1068" t="inlineStr">
         <is>
-          <t>Ana Milena Juan Davit</t>
+          <t>Ana Milena-Juan David</t>
         </is>
       </c>
       <c r="C1068" t="inlineStr">
@@ -34694,7 +34694,7 @@
       </c>
       <c r="B1069" t="inlineStr">
         <is>
-          <t>Ana Milena Juan Davit</t>
+          <t>Ana Milena-Juan David</t>
         </is>
       </c>
       <c r="C1069" t="inlineStr">
@@ -34725,7 +34725,7 @@
       </c>
       <c r="B1070" t="inlineStr">
         <is>
-          <t>Ana Milena Juan Davit</t>
+          <t>Ana Milena-Juan David</t>
         </is>
       </c>
       <c r="C1070" t="inlineStr">
@@ -34756,7 +34756,7 @@
       </c>
       <c r="B1071" t="inlineStr">
         <is>
-          <t>Ana Milena Juan Davit</t>
+          <t>Ana Milena-Juan David</t>
         </is>
       </c>
       <c r="C1071" t="inlineStr">
@@ -34787,7 +34787,7 @@
       </c>
       <c r="B1072" t="inlineStr">
         <is>
-          <t>Ana Milena Juan Davit</t>
+          <t>Ana Milena-Juan David</t>
         </is>
       </c>
       <c r="C1072" t="inlineStr">
@@ -34818,7 +34818,7 @@
       </c>
       <c r="B1073" t="inlineStr">
         <is>
-          <t>Ana Milena Juan Davit</t>
+          <t>Ana Milena-Juan David</t>
         </is>
       </c>
       <c r="C1073" t="inlineStr">
@@ -34849,7 +34849,7 @@
       </c>
       <c r="B1074" t="inlineStr">
         <is>
-          <t>Ana Milena Juan Davit</t>
+          <t>Ana Milena-Juan David</t>
         </is>
       </c>
       <c r="C1074" t="inlineStr">
@@ -34880,7 +34880,7 @@
       </c>
       <c r="B1075" t="inlineStr">
         <is>
-          <t>Ana Milena Juan Davit</t>
+          <t>Ana Milena-Juan David</t>
         </is>
       </c>
       <c r="C1075" t="inlineStr">
@@ -34911,7 +34911,7 @@
       </c>
       <c r="B1076" t="inlineStr">
         <is>
-          <t>Ana Milena Juan Davit</t>
+          <t>Ana Milena-Juan David</t>
         </is>
       </c>
       <c r="C1076" t="inlineStr">
@@ -34942,7 +34942,7 @@
       </c>
       <c r="B1077" t="inlineStr">
         <is>
-          <t>Ana Milena Juan Davit</t>
+          <t>Ana Milena-Juan David</t>
         </is>
       </c>
       <c r="C1077" t="inlineStr">
@@ -35407,7 +35407,7 @@
       </c>
       <c r="B1092" t="inlineStr">
         <is>
-          <t>Manuel Alga</t>
+          <t>Manuel Olga</t>
         </is>
       </c>
       <c r="C1092" t="inlineStr">
@@ -35438,7 +35438,7 @@
       </c>
       <c r="B1093" t="inlineStr">
         <is>
-          <t>Manuel Alga</t>
+          <t>Manuel Olga</t>
         </is>
       </c>
       <c r="C1093" t="inlineStr">
@@ -35469,7 +35469,7 @@
       </c>
       <c r="B1094" t="inlineStr">
         <is>
-          <t>Manuel Alga</t>
+          <t>Manuel Olga</t>
         </is>
       </c>
       <c r="C1094" t="inlineStr">
@@ -35500,7 +35500,7 @@
       </c>
       <c r="B1095" t="inlineStr">
         <is>
-          <t>Manuel Alga</t>
+          <t>Manuel Olga</t>
         </is>
       </c>
       <c r="C1095" t="inlineStr">
@@ -35531,7 +35531,7 @@
       </c>
       <c r="B1096" t="inlineStr">
         <is>
-          <t>Manuel Alga</t>
+          <t>Manuel Olga</t>
         </is>
       </c>
       <c r="C1096" t="inlineStr">
@@ -35562,7 +35562,7 @@
       </c>
       <c r="B1097" t="inlineStr">
         <is>
-          <t>Manuel Alga</t>
+          <t>Manuel Olga</t>
         </is>
       </c>
       <c r="C1097" t="inlineStr">
@@ -35593,7 +35593,7 @@
       </c>
       <c r="B1098" t="inlineStr">
         <is>
-          <t>Manuel Alga</t>
+          <t>Manuel Olga</t>
         </is>
       </c>
       <c r="C1098" t="inlineStr">
@@ -35624,7 +35624,7 @@
       </c>
       <c r="B1099" t="inlineStr">
         <is>
-          <t>Manuel Alga</t>
+          <t>Manuel Olga</t>
         </is>
       </c>
       <c r="C1099" t="inlineStr">
@@ -35655,7 +35655,7 @@
       </c>
       <c r="B1100" t="inlineStr">
         <is>
-          <t>Manuel Alga</t>
+          <t>Manuel Olga</t>
         </is>
       </c>
       <c r="C1100" t="inlineStr">
@@ -35686,7 +35686,7 @@
       </c>
       <c r="B1101" t="inlineStr">
         <is>
-          <t>Manuel Alga</t>
+          <t>Manuel Olga</t>
         </is>
       </c>
       <c r="C1101" t="inlineStr">
@@ -35717,7 +35717,7 @@
       </c>
       <c r="B1102" t="inlineStr">
         <is>
-          <t>Manuel Alga</t>
+          <t>Manuel Olga</t>
         </is>
       </c>
       <c r="C1102" t="inlineStr">
@@ -35748,7 +35748,7 @@
       </c>
       <c r="B1103" t="inlineStr">
         <is>
-          <t>Manuel Alga</t>
+          <t>Manuel Olga</t>
         </is>
       </c>
       <c r="C1103" t="inlineStr">
@@ -35779,7 +35779,7 @@
       </c>
       <c r="B1104" t="inlineStr">
         <is>
-          <t>Manuel Alga</t>
+          <t>Manuel Olga</t>
         </is>
       </c>
       <c r="C1104" t="inlineStr">
@@ -35810,7 +35810,7 @@
       </c>
       <c r="B1105" t="inlineStr">
         <is>
-          <t>Manuel Alga</t>
+          <t>Manuel Olga</t>
         </is>
       </c>
       <c r="C1105" t="inlineStr">
@@ -35841,7 +35841,7 @@
       </c>
       <c r="B1106" t="inlineStr">
         <is>
-          <t>Manuel Alga</t>
+          <t>Manuel Olga</t>
         </is>
       </c>
       <c r="C1106" t="inlineStr">
@@ -35872,7 +35872,7 @@
       </c>
       <c r="B1107" t="inlineStr">
         <is>
-          <t>Manuel Alga</t>
+          <t>Manuel Olga</t>
         </is>
       </c>
       <c r="C1107" t="inlineStr">
@@ -35903,7 +35903,7 @@
       </c>
       <c r="B1108" t="inlineStr">
         <is>
-          <t>Manuel Alga</t>
+          <t>Manuel Olga</t>
         </is>
       </c>
       <c r="C1108" t="inlineStr">
@@ -35934,7 +35934,7 @@
       </c>
       <c r="B1109" t="inlineStr">
         <is>
-          <t>Manuel Alga</t>
+          <t>Manuel Olga</t>
         </is>
       </c>
       <c r="C1109" t="inlineStr">
@@ -36461,7 +36461,7 @@
       </c>
       <c r="B1126" t="inlineStr">
         <is>
-          <t>Donita Juan Camilo</t>
+          <t>Daniela Nuñez</t>
         </is>
       </c>
       <c r="C1126" t="inlineStr">
@@ -36492,7 +36492,7 @@
       </c>
       <c r="B1127" t="inlineStr">
         <is>
-          <t>Donita Juan Camilo</t>
+          <t>Daniela Nuñez</t>
         </is>
       </c>
       <c r="C1127" t="inlineStr">
@@ -36523,7 +36523,7 @@
       </c>
       <c r="B1128" t="inlineStr">
         <is>
-          <t>Donita Juan Camilo</t>
+          <t>Daniela Nuñez</t>
         </is>
       </c>
       <c r="C1128" t="inlineStr">
@@ -36554,7 +36554,7 @@
       </c>
       <c r="B1129" t="inlineStr">
         <is>
-          <t>Donita Juan Camilo</t>
+          <t>Daniela Nuñez</t>
         </is>
       </c>
       <c r="C1129" t="inlineStr">
@@ -36585,7 +36585,7 @@
       </c>
       <c r="B1130" t="inlineStr">
         <is>
-          <t>Alejandra</t>
+          <t>Alejandro</t>
         </is>
       </c>
       <c r="C1130" t="inlineStr">
@@ -36616,7 +36616,7 @@
       </c>
       <c r="B1131" t="inlineStr">
         <is>
-          <t>Alejandra</t>
+          <t>Alejandro</t>
         </is>
       </c>
       <c r="C1131" t="inlineStr">
@@ -36647,7 +36647,7 @@
       </c>
       <c r="B1132" t="inlineStr">
         <is>
-          <t>Alejandra</t>
+          <t>Alejandro</t>
         </is>
       </c>
       <c r="C1132" t="inlineStr">
@@ -36678,7 +36678,7 @@
       </c>
       <c r="B1133" t="inlineStr">
         <is>
-          <t>Alejandra</t>
+          <t>Alejandro</t>
         </is>
       </c>
       <c r="C1133" t="inlineStr">
@@ -36709,7 +36709,7 @@
       </c>
       <c r="B1134" t="inlineStr">
         <is>
-          <t>Alejandra</t>
+          <t>Alejandro</t>
         </is>
       </c>
       <c r="C1134" t="inlineStr">
@@ -36740,7 +36740,7 @@
       </c>
       <c r="B1135" t="inlineStr">
         <is>
-          <t>Alejandra</t>
+          <t>Alejandro</t>
         </is>
       </c>
       <c r="C1135" t="inlineStr">
@@ -36771,7 +36771,7 @@
       </c>
       <c r="B1136" t="inlineStr">
         <is>
-          <t>Alejandra</t>
+          <t>Alejandro</t>
         </is>
       </c>
       <c r="C1136" t="inlineStr">
@@ -36802,7 +36802,7 @@
       </c>
       <c r="B1137" t="inlineStr">
         <is>
-          <t>Alejandra</t>
+          <t>Alejandro</t>
         </is>
       </c>
       <c r="C1137" t="inlineStr">
@@ -36833,7 +36833,7 @@
       </c>
       <c r="B1138" t="inlineStr">
         <is>
-          <t>Alejandra</t>
+          <t>Alejandro</t>
         </is>
       </c>
       <c r="C1138" t="inlineStr">
@@ -36864,7 +36864,7 @@
       </c>
       <c r="B1139" t="inlineStr">
         <is>
-          <t>Alejandra</t>
+          <t>Alejandro</t>
         </is>
       </c>
       <c r="C1139" t="inlineStr">
@@ -36895,7 +36895,7 @@
       </c>
       <c r="B1140" t="inlineStr">
         <is>
-          <t>Alejandra</t>
+          <t>Alejandro</t>
         </is>
       </c>
       <c r="C1140" t="inlineStr">
@@ -36926,7 +36926,7 @@
       </c>
       <c r="B1141" t="inlineStr">
         <is>
-          <t>Alejandra</t>
+          <t>Alejandro</t>
         </is>
       </c>
       <c r="C1141" t="inlineStr">
@@ -36957,7 +36957,7 @@
       </c>
       <c r="B1142" t="inlineStr">
         <is>
-          <t>Alejandra</t>
+          <t>Alejandro</t>
         </is>
       </c>
       <c r="C1142" t="inlineStr">
@@ -36988,7 +36988,7 @@
       </c>
       <c r="B1143" t="inlineStr">
         <is>
-          <t>Carlos</t>
+          <t>Karluis</t>
         </is>
       </c>
       <c r="C1143" t="inlineStr">
@@ -37019,7 +37019,7 @@
       </c>
       <c r="B1144" t="inlineStr">
         <is>
-          <t>Carlos</t>
+          <t>Karluis</t>
         </is>
       </c>
       <c r="C1144" t="inlineStr">
@@ -37050,7 +37050,7 @@
       </c>
       <c r="B1145" t="inlineStr">
         <is>
-          <t>Carlos</t>
+          <t>Karluis</t>
         </is>
       </c>
       <c r="C1145" t="inlineStr">
@@ -37081,7 +37081,7 @@
       </c>
       <c r="B1146" t="inlineStr">
         <is>
-          <t>Carlos</t>
+          <t>Karluis</t>
         </is>
       </c>
       <c r="C1146" t="inlineStr">

</xml_diff>

<commit_message>
feat: calculadora inversa de intereses en dashboard y Excel
- Dashboard (Creditos): nueva seccion 'Que interes le estoy cobrando?'
  Modo A: ingresa valor moto + total a cobrar + meses -> cuota y % interes
  Modo B: ingresa valor moto + cuota mensual + meses -> total y % interes
  Calculo usa formula compuesta (RATE / biseccion Newton)
- Excel (Simulador): misma calculadora en filas 105-125 de la hoja Simulador

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/control_motos_tio.xlsx
+++ b/control_motos_tio.xlsx
@@ -18,11 +18,12 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
     <numFmt numFmtId="165" formatCode="DD/MM/YYYY"/>
+    <numFmt numFmtId="166" formatCode="0.00 &quot;%&quot;"/>
   </numFmts>
-  <fonts count="11">
+  <fonts count="13">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -75,8 +76,18 @@
       <color rgb="00555555"/>
       <sz val="9"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00F4EFE2"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="007B3F00"/>
+      <sz val="12"/>
+    </font>
   </fonts>
-  <fills count="11">
+  <fills count="12">
     <fill>
       <patternFill/>
     </fill>
@@ -128,6 +139,11 @@
         <fgColor rgb="00F8F9FA"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="007B3F00"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -147,7 +163,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -199,6 +215,18 @@
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="11" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="12" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1189,7 +1217,7 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>Amigo de Guillo | 21 meses | 20160000 total | 84 cuotas | subtotal cuaderno ~11.280.000 (≈47 cuotas) | algunos pagos son multiples por fila</t>
+          <t>Amigo de Guillo | 21 meses | 20160000 total | 84 cuotas | subtotal cuaderno ~11.280.000 (~47 cuotas) | algunos pagos son multiples por fila</t>
         </is>
       </c>
       <c r="F22" t="n">
@@ -37396,7 +37424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F102"/>
+  <dimension ref="A1:F125"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -39678,15 +39706,208 @@
     <row r="102">
       <c r="A102" s="19" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Celdas amarillas → entrada manual  |  Celdas verdes → calculadas automáticamente</t>
+          <t xml:space="preserve">  Celdas amarillas -&gt; entrada manual  |  Celdas verdes -&gt; calculadas automáticamente</t>
+        </is>
+      </c>
+    </row>
+    <row r="104" ht="16" customHeight="1"/>
+    <row r="105" ht="34" customHeight="1">
+      <c r="A105" s="20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  CALCULADORA INVERSA  —  ¿Qué interés le estoy cobrando al cliente?</t>
+        </is>
+      </c>
+    </row>
+    <row r="106" ht="8" customHeight="1"/>
+    <row r="107" ht="22" customHeight="1">
+      <c r="A107" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Modo A · Conozco el TOTAL que quiero cobrar</t>
+        </is>
+      </c>
+    </row>
+    <row r="108" ht="24" customHeight="1">
+      <c r="A108" s="6" t="inlineStr">
+        <is>
+          <t>Valor de la moto  (lo que presté)</t>
+        </is>
+      </c>
+      <c r="B108" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="C108" s="8" t="inlineStr">
+        <is>
+          <t>← capital prestado al cliente</t>
+        </is>
+      </c>
+    </row>
+    <row r="109" ht="24" customHeight="1">
+      <c r="A109" s="6" t="inlineStr">
+        <is>
+          <t>Total que quiero cobrar  ($)</t>
+        </is>
+      </c>
+      <c r="B109" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="C109" s="8" t="inlineStr">
+        <is>
+          <t>← suma total que quieres recibir</t>
+        </is>
+      </c>
+    </row>
+    <row r="110" ht="24" customHeight="1">
+      <c r="A110" s="6" t="inlineStr">
+        <is>
+          <t>Número de meses</t>
+        </is>
+      </c>
+      <c r="B110" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="C110" s="8" t="inlineStr">
+        <is>
+          <t>← duración del crédito</t>
+        </is>
+      </c>
+    </row>
+    <row r="111" ht="8" customHeight="1"/>
+    <row r="112" ht="26" customHeight="1">
+      <c r="A112" s="12" t="inlineStr">
+        <is>
+          <t>Cuota mensual</t>
+        </is>
+      </c>
+      <c r="B112" s="13">
+        <f>IFERROR(B109/B110,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="113" ht="26" customHeight="1">
+      <c r="A113" s="12" t="inlineStr">
+        <is>
+          <t>Interés mensual  (%)</t>
+        </is>
+      </c>
+      <c r="B113" s="23">
+        <f>IFERROR(RATE(B110,-B112,B108)*100,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="114" ht="26" customHeight="1">
+      <c r="A114" s="12" t="inlineStr">
+        <is>
+          <t>Interés anual  (%)</t>
+        </is>
+      </c>
+      <c r="B114" s="23">
+        <f>IFERROR(B113*12,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="115" ht="14" customHeight="1"/>
+    <row r="116" ht="22" customHeight="1">
+      <c r="A116" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Modo B · Conozco la CUOTA mensual que le voy a cobrar</t>
+        </is>
+      </c>
+    </row>
+    <row r="117" ht="24" customHeight="1">
+      <c r="A117" s="6" t="inlineStr">
+        <is>
+          <t>Valor de la moto  (lo que presté)</t>
+        </is>
+      </c>
+      <c r="B117" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="C117" s="8" t="inlineStr">
+        <is>
+          <t>← capital prestado al cliente</t>
+        </is>
+      </c>
+    </row>
+    <row r="118" ht="24" customHeight="1">
+      <c r="A118" s="6" t="inlineStr">
+        <is>
+          <t>Cuota mensual  ($)</t>
+        </is>
+      </c>
+      <c r="B118" s="21" t="n">
+        <v>0</v>
+      </c>
+      <c r="C118" s="8" t="inlineStr">
+        <is>
+          <t>← cuánto va a pagar cada mes</t>
+        </is>
+      </c>
+    </row>
+    <row r="119" ht="24" customHeight="1">
+      <c r="A119" s="6" t="inlineStr">
+        <is>
+          <t>Número de meses</t>
+        </is>
+      </c>
+      <c r="B119" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="C119" s="8" t="inlineStr">
+        <is>
+          <t>← duración del crédito</t>
+        </is>
+      </c>
+    </row>
+    <row r="120" ht="8" customHeight="1"/>
+    <row r="121" ht="26" customHeight="1">
+      <c r="A121" s="12" t="inlineStr">
+        <is>
+          <t>Total a cobrar  ($)</t>
+        </is>
+      </c>
+      <c r="B121" s="13">
+        <f>IFERROR(B118*B119,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="122" ht="26" customHeight="1">
+      <c r="A122" s="12" t="inlineStr">
+        <is>
+          <t>Interés mensual  (%)</t>
+        </is>
+      </c>
+      <c r="B122" s="23">
+        <f>IFERROR(RATE(B119,-B118,B117)*100,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="123" ht="26" customHeight="1">
+      <c r="A123" s="12" t="inlineStr">
+        <is>
+          <t>Interés anual  (%)</t>
+        </is>
+      </c>
+      <c r="B123" s="23">
+        <f>IFERROR(B122*12,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" s="19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Celdas amarillas -&gt; entrada manual  |  Celdas verdes -&gt; calculadas  |  Interés usa fórmula compuesta (RATE de Excel)</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="5">
+  <mergeCells count="9">
+    <mergeCell ref="A125:F125"/>
+    <mergeCell ref="A107:F107"/>
     <mergeCell ref="A102:F102"/>
     <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A116:F116"/>
     <mergeCell ref="A9:F9"/>
+    <mergeCell ref="A105:F105"/>
     <mergeCell ref="A3:F3"/>
     <mergeCell ref="A15:F15"/>
   </mergeCells>

</xml_diff>

<commit_message>
Leer teléfonos desde columna G del Excel (cruce por placa)
- cargar_clientes() ahora lee col G (Telefono conductor) y valida
  solo números móviles colombianos (10 dígitos, empieza en 3)
- Retorna también tel_por_placa para cruce exacto placa→tel
- procesar() acepta tel_por_placa como fuente primaria de teléfono
- Prioridad: placa Excel > nombre meta > CLIENTES_CONFIG tel
- negro luis y edinson ahora reciben su número vía placa
- 13 clientes con botón SMS activo

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/control_motos_tio.xlsx
+++ b/control_motos_tio.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jeffer\Desktop\motos-tio-master\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8C9B0B87-4C4E-4474-9840-59DE17097099}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{99AF78F3-3D21-42DE-A094-561DDC507033}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-104" yWindow="-104" windowWidth="22326" windowHeight="11947" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-104" yWindow="-104" windowWidth="22326" windowHeight="11947" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Clientes" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4545" uniqueCount="208">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4544" uniqueCount="207">
   <si>
     <t>Nombre</t>
   </si>
@@ -660,9 +660,6 @@
   <si>
     <t>no tiene</t>
   </si>
-  <si>
-    <t>*48513310431</t>
-  </si>
 </sst>
 </file>
 
@@ -847,7 +844,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="37">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -941,8 +938,6 @@
     <xf numFmtId="0" fontId="11" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="13" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="164" fontId="0" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1592,8 +1587,8 @@
       <c r="F14" s="27">
         <v>84</v>
       </c>
-      <c r="G14" s="27" t="s">
-        <v>207</v>
+      <c r="G14" s="27">
+        <v>48513310431</v>
       </c>
     </row>
     <row r="15" spans="1:13" s="27" customFormat="1" x14ac:dyDescent="0.3">
@@ -1665,26 +1660,26 @@
         <v>3235367102</v>
       </c>
     </row>
-    <row r="18" spans="1:7" s="35" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="35" t="s">
+    <row r="18" spans="1:7" s="27" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A18" s="27" t="s">
         <v>70</v>
       </c>
-      <c r="B18" s="35" t="s">
+      <c r="B18" s="27" t="s">
         <v>71</v>
       </c>
-      <c r="C18" s="35" t="s">
+      <c r="C18" s="27" t="s">
         <v>72</v>
       </c>
-      <c r="D18" s="36">
+      <c r="D18" s="28">
         <v>45832</v>
       </c>
-      <c r="E18" s="35" t="s">
+      <c r="E18" s="27" t="s">
         <v>73</v>
       </c>
-      <c r="F18" s="35">
+      <c r="F18" s="27">
         <v>64</v>
       </c>
-      <c r="G18" s="35">
+      <c r="G18" s="27">
         <v>3017355501</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Actualizar dashboard — teléfonos Erick y Juan David/Ana Milena
</commit_message>
<xml_diff>
--- a/control_motos_tio.xlsx
+++ b/control_motos_tio.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jeffer\Desktop\motos-tio-master\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{178864A8-6C53-4BAB-8EC8-14C955F29651}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{52497D56-8813-44CD-84DA-58F0299A8AAA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3030" yWindow="887" windowWidth="16589" windowHeight="10898" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-104" yWindow="-104" windowWidth="22326" windowHeight="11947" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Clientes" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4571" uniqueCount="214">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4572" uniqueCount="214">
   <si>
     <t>Nombre</t>
   </si>
@@ -704,68 +704,80 @@
       <sz val="11"/>
       <color rgb="FFF4EFE2"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="16"/>
       <color rgb="FFF4EFE2"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="11"/>
       <color rgb="FFF4EFE2"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="10"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="11"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <i/>
       <sz val="9"/>
       <color rgb="FF888888"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="12"/>
       <color rgb="FF1B4332"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="10"/>
       <color rgb="FFFFFFFF"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="9"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <i/>
       <sz val="9"/>
       <color rgb="FF555555"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="14"/>
       <color rgb="FFF4EFE2"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="12"/>
       <color rgb="FF7B3F00"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="14">
@@ -865,7 +877,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="37">
+  <cellXfs count="38">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -960,6 +972,9 @@
     </xf>
     <xf numFmtId="0" fontId="11" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="12" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1771,6 +1786,9 @@
       <c r="F21" s="27">
         <v>36</v>
       </c>
+      <c r="G21" s="37">
+        <v>3245613478</v>
+      </c>
     </row>
     <row r="22" spans="1:7" s="27" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A22" s="27" t="s">
@@ -1838,7 +1856,7 @@
         <v>64</v>
       </c>
       <c r="G24" s="27">
-        <v>3004635466</v>
+        <v>3021121287</v>
       </c>
     </row>
     <row r="25" spans="1:7" s="27" customFormat="1" x14ac:dyDescent="0.3">
@@ -2091,20 +2109,20 @@
         <v>207</v>
       </c>
     </row>
-    <row r="36" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:8" s="27" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A36" s="27" t="s">
         <v>212</v>
       </c>
       <c r="C36" s="27" t="s">
         <v>213</v>
       </c>
-      <c r="E36">
-        <v>260</v>
+      <c r="E36" s="27" t="s">
+        <v>208</v>
       </c>
       <c r="F36" s="27">
         <v>48</v>
       </c>
-      <c r="H36" t="s">
+      <c r="H36" s="27" t="s">
         <v>207</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Gustavo Primo: corregir pago 22/08 a 480k (2 cuotas de 240k)
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/control_motos_tio.xlsx
+++ b/control_motos_tio.xlsx
@@ -35785,7 +35785,7 @@
         <v>240000</v>
       </c>
       <c r="I1094" t="n">
-        <v>180000</v>
+        <v>240000</v>
       </c>
       <c r="J1094" t="inlineStr">
         <is>
@@ -35794,7 +35794,7 @@
       </c>
       <c r="P1094" t="inlineStr">
         <is>
-          <t>pago conjunto 420k (2 cuotas)</t>
+          <t>pago conjunto 480k (2 cuotas)</t>
         </is>
       </c>
     </row>

</xml_diff>